<commit_message>
alpha energy relative error
</commit_message>
<xml_diff>
--- a/testResults/timestepStabilityResults/timestepStabilityResults.xlsx
+++ b/testResults/timestepStabilityResults/timestepStabilityResults.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t xml:space="preserve">Max Stability Time</t>
   </si>
@@ -27,7 +27,7 @@
     <t>T</t>
   </si>
   <si>
-    <t xml:space="preserve">Relative Error</t>
+    <t xml:space="preserve">Relative Error Phi</t>
   </si>
   <si>
     <t>DT</t>
@@ -37,6 +37,12 @@
   </si>
   <si>
     <t xml:space="preserve">Max Resolved Time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relative Error E_alpha</t>
+  </si>
+  <si>
+    <t>Resol</t>
   </si>
   <si>
     <t>Alpha</t>
@@ -78,10 +84,16 @@
     <t>~1E-1</t>
   </si>
   <si>
+    <t>~1E-3</t>
+  </si>
+  <si>
     <t>2^-4</t>
   </si>
   <si>
     <t>~1E-2</t>
+  </si>
+  <si>
+    <t>~1E-4</t>
   </si>
   <si>
     <t>2^-5</t>
@@ -90,13 +102,13 @@
     <t>stable</t>
   </si>
   <si>
-    <t>~1E-3</t>
+    <t>~1E-5</t>
   </si>
   <si>
     <t>2^-6</t>
   </si>
   <si>
-    <t>~1E-4</t>
+    <t>~1E-6</t>
   </si>
   <si>
     <t>2^-7</t>
@@ -105,7 +117,16 @@
     <t>~1E-(5-9)</t>
   </si>
   <si>
+    <t>~1E-(7-9)</t>
+  </si>
+  <si>
     <t>&lt;1E-10</t>
+  </si>
+  <si>
+    <t>&lt;1E-9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relative Error</t>
   </si>
 </sst>
 </file>
@@ -120,7 +141,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -171,14 +192,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor theme="6" tint="0.39997558519241921"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="5" tint="-0.249977111117893"/>
         <bgColor theme="5" tint="-0.249977111117893"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
-        <bgColor theme="6" tint="0.39997558519241921"/>
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor theme="4" tint="0.39997558519241921"/>
       </patternFill>
     </fill>
     <fill>
@@ -188,7 +215,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="29">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -213,6 +240,15 @@
     </border>
     <border>
       <left style="none"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
       <right style="none"/>
       <top style="none"/>
       <bottom style="thin">
@@ -234,12 +270,14 @@
       <diagonal style="none"/>
     </border>
     <border>
-      <left style="none"/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="none"/>
       <top style="none"/>
-      <bottom style="none"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal style="none"/>
     </border>
     <border>
@@ -328,6 +366,21 @@
       </left>
       <right style="thin">
         <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
       </right>
       <top style="thin">
         <color auto="1"/>
@@ -379,11 +432,56 @@
       <diagonal style="none"/>
     </border>
     <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
       <left style="none"/>
       <right style="thin">
         <color auto="1"/>
       </right>
       <top style="none"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -435,26 +533,13 @@
       <diagonal style="none"/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
+      <left style="none"/>
       <right style="thin">
         <color auto="1"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color theme="1"/>
       </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="none"/>
-      <top style="none"/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -514,7 +599,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="79">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
@@ -524,79 +609,98 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
-      <protection hidden="0" locked="1"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="0" fillId="2" borderId="3" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1">
+    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1">
       <protection hidden="0" locked="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="0" fillId="2" borderId="4" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="2" borderId="5" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="3" borderId="6" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="5" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="0" fillId="2" borderId="6" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="3" borderId="7" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="3" borderId="8" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="3" borderId="9" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="6" borderId="1" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="9" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="10" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="0" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1">
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="0" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1">
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="10" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="8" borderId="1" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="9" borderId="1" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="3" borderId="11" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="4" borderId="8" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="3" borderId="3" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="3" borderId="12" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="4" borderId="9" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="3" borderId="4" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="3" borderId="13" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="10" borderId="1" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="11" borderId="1" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="4" borderId="14" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="10" borderId="15" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="10" borderId="16" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="8" borderId="9" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="10" borderId="17" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="10" borderId="16" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="10" borderId="18" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="8" borderId="19" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="10" borderId="7" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="8" borderId="14" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="9" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="4" borderId="12" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="9" borderId="13" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="9" borderId="14" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="8" borderId="8" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="10" borderId="1" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="8" borderId="15" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="8" borderId="12" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf fontId="0" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="10" borderId="20" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="9" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="11" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
-    <xf fontId="0" fillId="11" borderId="0" numFmtId="0" xfId="0" applyFill="1">
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="3" borderId="14" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="3" borderId="16" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="3" borderId="17" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="4" borderId="15" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="3" borderId="18" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="2" borderId="19" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="20" numFmtId="0" xfId="0" applyBorder="1">
+    <xf fontId="0" fillId="12" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
+    <xf fontId="0" fillId="12" borderId="0" numFmtId="0" xfId="0" applyFill="1">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="2" borderId="21" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="3" borderId="16" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="3" borderId="21" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="3" borderId="22" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="4" borderId="19" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="8" borderId="15" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="11" borderId="18" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="8" borderId="17" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="8" borderId="7" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="8" borderId="20" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="3" borderId="23" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="3" borderId="24" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="9" numFmtId="0" xfId="0" applyBorder="1">
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="5" borderId="18" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="5" borderId="24" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="2" borderId="13" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="5" numFmtId="0" xfId="0" applyBorder="1">
       <protection hidden="0" locked="1"/>
     </xf>
+    <xf fontId="0" fillId="2" borderId="25" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="3" borderId="26" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="3" borderId="27" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="3" borderId="28" numFmtId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="10" numFmtId="0" xfId="0" applyBorder="1">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="20" numFmtId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1135,10 +1239,10 @@
         <v>5</v>
       </c>
       <c r="S1" s="3"/>
-      <c r="T1" s="4" t="s">
+      <c r="T1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="U1" s="5"/>
+      <c r="U1" s="3"/>
       <c r="V1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1151,41 +1255,77 @@
       <c r="Y1" s="2">
         <v>5</v>
       </c>
-      <c r="Z1" s="4"/>
+      <c r="Z1" s="3"/>
+      <c r="AB1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="AC1" s="5"/>
+      <c r="AD1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AE1" s="2">
+        <v>128</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="AG1" s="2">
+        <v>5</v>
+      </c>
+      <c r="AH1" s="3"/>
+      <c r="AI1" s="3"/>
     </row>
     <row r="2" ht="14.25">
-      <c r="S2" s="4"/>
-      <c r="T2" s="4"/>
-      <c r="U2" s="4"/>
-      <c r="V2" s="4"/>
-      <c r="W2" s="4"/>
-      <c r="X2" s="4"/>
-      <c r="Y2" s="4"/>
-      <c r="Z2" s="4"/>
+      <c r="S2" s="3"/>
+      <c r="T2" s="3"/>
+      <c r="U2" s="3"/>
+      <c r="V2" s="3"/>
+      <c r="W2" s="3"/>
+      <c r="X2" s="3"/>
+      <c r="Y2" s="3"/>
+      <c r="Z2" s="3"/>
+      <c r="AB2" s="3"/>
+      <c r="AC2" s="3"/>
+      <c r="AD2" s="3"/>
+      <c r="AE2" s="3"/>
+      <c r="AF2" s="3"/>
+      <c r="AG2" s="3"/>
+      <c r="AH2" s="3"/>
+      <c r="AI2" s="3"/>
     </row>
     <row r="3" ht="14.25">
       <c r="D3" t="s">
-        <v>7</v>
-      </c>
-      <c r="J3" s="4"/>
+        <v>9</v>
+      </c>
+      <c r="J3" s="3"/>
       <c r="K3" s="6"/>
       <c r="L3" s="6"/>
       <c r="M3" s="7" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N3" s="6"/>
       <c r="O3" s="6"/>
       <c r="P3" s="6"/>
-      <c r="S3" s="4"/>
+      <c r="S3" s="3"/>
       <c r="T3" s="6"/>
       <c r="U3" s="6"/>
       <c r="V3" s="7" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="W3" s="6"/>
       <c r="X3" s="6"/>
       <c r="Y3" s="6"/>
-      <c r="Z3" s="4"/>
+      <c r="Z3" s="3"/>
+      <c r="AB3" s="3"/>
+      <c r="AC3" s="6"/>
+      <c r="AD3" s="6"/>
+      <c r="AE3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="AF3" s="6"/>
+      <c r="AG3" s="6"/>
+      <c r="AH3" s="6"/>
+      <c r="AI3" s="3"/>
     </row>
     <row r="4" ht="14.25">
       <c r="B4" s="1"/>
@@ -1204,49 +1344,67 @@
       <c r="G4" s="1">
         <v>16</v>
       </c>
-      <c r="J4" s="9"/>
+      <c r="J4" s="5"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q4" s="10"/>
-      <c r="R4" s="10"/>
-      <c r="S4" s="9"/>
+        <v>14</v>
+      </c>
+      <c r="Q4" s="9"/>
+      <c r="R4" s="9"/>
+      <c r="S4" s="5"/>
       <c r="T4" s="1"/>
       <c r="U4" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="V4" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="W4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="X4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="Y4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Z4" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="AB4" s="5"/>
+      <c r="AC4" s="1"/>
+      <c r="AD4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="X4" s="1" t="s">
+      <c r="AE4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="Y4" s="1" t="s">
+      <c r="AF4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="11" t="s">
+      <c r="AG4" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="AH4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="AI4" s="11"/>
     </row>
     <row r="5" ht="14.25">
       <c r="B5" s="12" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C5" s="13">
         <v>2.75</v>
@@ -1263,57 +1421,79 @@
       <c r="G5" s="16">
         <v>5</v>
       </c>
-      <c r="J5" s="9"/>
+      <c r="J5" s="5"/>
       <c r="K5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="L5" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="M5" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="N5" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="O5" s="18">
+        <v>16</v>
+      </c>
+      <c r="L5" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M5" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N5" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="O5" s="17">
         <v>0.0044999999999999997</v>
       </c>
-      <c r="P5" s="19">
+      <c r="P5" s="18">
         <v>6.9999999999999994e-05</v>
       </c>
-      <c r="Q5" s="17" t="s">
+      <c r="Q5" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="R5" s="19"/>
+      <c r="S5" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="T5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="U5" s="21">
+        <v>2.4375</v>
+      </c>
+      <c r="V5" s="21">
+        <v>2.55878125</v>
+      </c>
+      <c r="W5" s="21">
+        <v>2.859375</v>
+      </c>
+      <c r="X5" s="21">
+        <v>3.671875</v>
+      </c>
+      <c r="Y5" s="22">
+        <v>5</v>
+      </c>
+      <c r="Z5" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="AB5" s="5"/>
+      <c r="AC5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R5" s="20"/>
-      <c r="S5" s="21" t="s">
-        <v>4</v>
-      </c>
-      <c r="T5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="U5" s="22">
-        <v>2.4375</v>
-      </c>
-      <c r="V5" s="22">
-        <v>2.55878125</v>
-      </c>
-      <c r="W5" s="22">
-        <v>2.859375</v>
-      </c>
-      <c r="X5" s="22">
-        <v>3.671875</v>
-      </c>
-      <c r="Y5" s="23">
-        <v>5</v>
-      </c>
-      <c r="Z5" s="24" t="s">
-        <v>17</v>
+      <c r="AD5" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE5" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF5" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG5" s="23">
+        <v>0.00038200000000000002</v>
+      </c>
+      <c r="AH5" s="24">
+        <v>8.7299999999999994e-06</v>
+      </c>
+      <c r="AI5" s="10" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="6" ht="14.25">
       <c r="B6" s="12" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C6" s="25">
         <v>2.625</v>
@@ -1330,46 +1510,67 @@
       <c r="G6" s="16">
         <v>5</v>
       </c>
-      <c r="J6" s="21"/>
+      <c r="J6" s="20"/>
       <c r="K6" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="L6" s="28" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="M6" s="28" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="N6" s="29">
         <v>0.057200000000000001</v>
       </c>
-      <c r="O6" s="18">
+      <c r="O6" s="17">
         <v>0.0011000000000000001</v>
       </c>
-      <c r="P6" s="19">
+      <c r="P6" s="18">
         <v>3.6399999999999999e-06</v>
       </c>
       <c r="Q6" s="30" t="s">
-        <v>19</v>
-      </c>
-      <c r="R6" s="20"/>
-      <c r="S6"/>
-      <c r="T6" s="31"/>
-      <c r="U6" s="10"/>
-      <c r="V6" s="10"/>
-      <c r="W6" s="10"/>
-      <c r="X6" s="10"/>
-      <c r="Y6" s="10"/>
-      <c r="Z6" s="10"/>
+        <v>21</v>
+      </c>
+      <c r="R6" s="19"/>
+      <c r="T6" s="9"/>
+      <c r="U6" s="9"/>
+      <c r="V6" s="9"/>
+      <c r="W6" s="9"/>
+      <c r="X6" s="9"/>
+      <c r="Y6" s="9"/>
+      <c r="Z6" s="9"/>
+      <c r="AB6" s="20"/>
+      <c r="AC6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="AD6" s="31" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE6" s="31" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF6" s="32">
+        <v>0.0019400000000000001</v>
+      </c>
+      <c r="AG6" s="33">
+        <v>6.9099999999999999e-05</v>
+      </c>
+      <c r="AH6" s="18">
+        <v>3.72e-07</v>
+      </c>
+      <c r="AI6" s="34" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="7" ht="14.25">
       <c r="B7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="32">
-        <v>5</v>
-      </c>
-      <c r="D7" s="32">
+        <v>23</v>
+      </c>
+      <c r="C7" s="35">
+        <v>5</v>
+      </c>
+      <c r="D7" s="35">
         <v>5</v>
       </c>
       <c r="E7" s="16">
@@ -1381,48 +1582,69 @@
       <c r="G7" s="16">
         <v>5</v>
       </c>
-      <c r="H7" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="I7"/>
-      <c r="J7" s="5"/>
+      <c r="H7" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="J7" s="3"/>
       <c r="K7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="L7" s="33">
+        <v>23</v>
+      </c>
+      <c r="L7" s="36">
         <v>0.16619999999999999</v>
       </c>
-      <c r="M7" s="34">
+      <c r="M7" s="37">
         <v>0.1157</v>
       </c>
-      <c r="N7" s="35">
+      <c r="N7" s="38">
         <v>0.0332</v>
       </c>
-      <c r="O7" s="36">
+      <c r="O7" s="24">
         <v>0.00048480000000000002</v>
       </c>
-      <c r="P7" s="19">
+      <c r="P7" s="18">
         <v>2.0200000000000001e-07</v>
       </c>
       <c r="Q7" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="R7" s="20"/>
-      <c r="S7" s="4"/>
-      <c r="T7" s="31"/>
-      <c r="U7" s="10"/>
-      <c r="V7" s="10"/>
-      <c r="W7" s="10"/>
-      <c r="X7" s="10"/>
-      <c r="Y7" s="10"/>
-      <c r="Z7" s="10"/>
+        <v>24</v>
+      </c>
+      <c r="R7" s="19"/>
+      <c r="S7" s="3"/>
+      <c r="T7" s="9"/>
+      <c r="U7" s="9"/>
+      <c r="V7" s="9"/>
+      <c r="W7" s="9"/>
+      <c r="X7" s="9"/>
+      <c r="Y7" s="9"/>
+      <c r="Z7" s="9"/>
+      <c r="AB7" s="5"/>
+      <c r="AC7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="AD7" s="39">
+        <v>0.0033800000000000002</v>
+      </c>
+      <c r="AE7" s="40">
+        <v>0.0027399999999999998</v>
+      </c>
+      <c r="AF7" s="41">
+        <v>0.0011100000000000001</v>
+      </c>
+      <c r="AG7" s="33">
+        <v>3.0499999999999999e-05</v>
+      </c>
+      <c r="AH7" s="18">
+        <v>1.7599999999999999e-08</v>
+      </c>
+      <c r="AI7" s="42" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="8" ht="14.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C8" s="16">
         <v>5</v>
@@ -1439,47 +1661,70 @@
       <c r="G8" s="16">
         <v>5</v>
       </c>
-      <c r="H8" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="I8" s="4"/>
-      <c r="J8" s="31" t="s">
+      <c r="H8" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="I8" s="3"/>
+      <c r="J8" s="9" t="s">
         <v>4</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="L8" s="33">
+        <v>26</v>
+      </c>
+      <c r="L8" s="36">
         <v>0.10929999999999999</v>
       </c>
-      <c r="M8" s="37">
+      <c r="M8" s="43">
         <v>0.071499999999999994</v>
       </c>
       <c r="N8" s="29">
         <v>0.018100000000000002</v>
       </c>
-      <c r="O8" s="36">
+      <c r="O8" s="24">
         <v>0.000233</v>
       </c>
-      <c r="P8" s="19">
+      <c r="P8" s="18">
         <v>1.2100000000000001e-08</v>
       </c>
-      <c r="Q8" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="R8" s="20"/>
-      <c r="S8"/>
-      <c r="T8" s="31"/>
-      <c r="U8" s="10"/>
-      <c r="V8" s="10"/>
-      <c r="W8" s="10"/>
-      <c r="X8" s="10"/>
-      <c r="Y8" s="10"/>
-      <c r="Z8" s="4"/>
+      <c r="Q8" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="R8" s="19"/>
+      <c r="T8" s="9"/>
+      <c r="U8" s="9"/>
+      <c r="V8" s="9"/>
+      <c r="W8" s="9"/>
+      <c r="X8" s="9"/>
+      <c r="Y8" s="9"/>
+      <c r="Z8" s="3"/>
+      <c r="AB8" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="AC8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AD8" s="39">
+        <v>0.0023800000000000002</v>
+      </c>
+      <c r="AE8" s="44">
+        <v>0.00181</v>
+      </c>
+      <c r="AF8" s="23">
+        <v>0.00064899999999999995</v>
+      </c>
+      <c r="AG8" s="33">
+        <v>1.5699999999999999e-05</v>
+      </c>
+      <c r="AH8" s="45">
+        <v>9.590000000000001e-10</v>
+      </c>
+      <c r="AI8" s="46" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="9" ht="14.25">
       <c r="B9" s="1" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C9" s="16">
         <v>5</v>
@@ -1496,41 +1741,63 @@
       <c r="G9" s="16">
         <v>5</v>
       </c>
-      <c r="J9" s="9"/>
+      <c r="J9" s="5"/>
       <c r="K9" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="L9" s="38">
+        <v>29</v>
+      </c>
+      <c r="L9" s="47">
         <v>0.059299999999999999</v>
       </c>
       <c r="M9" s="29">
         <v>0.036900000000000002</v>
       </c>
-      <c r="N9" s="18">
+      <c r="N9" s="17">
         <v>0.0085000000000000006</v>
       </c>
-      <c r="O9" s="36">
+      <c r="O9" s="24">
         <v>0.000102</v>
       </c>
-      <c r="P9" s="39">
+      <c r="P9" s="45">
         <v>8.6300000000000002e-10</v>
       </c>
-      <c r="Q9" s="40" t="s">
-        <v>26</v>
-      </c>
-      <c r="R9" s="20"/>
-      <c r="S9" s="4"/>
-      <c r="T9" s="31"/>
-      <c r="U9" s="4"/>
-      <c r="V9" s="4"/>
-      <c r="W9" s="4"/>
-      <c r="X9" s="4"/>
-      <c r="Y9" s="4"/>
-      <c r="Z9" s="10"/>
+      <c r="Q9" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="R9" s="19"/>
+      <c r="S9" s="3"/>
+      <c r="T9" s="9"/>
+      <c r="U9" s="3"/>
+      <c r="V9" s="3"/>
+      <c r="W9" s="3"/>
+      <c r="X9" s="3"/>
+      <c r="Y9" s="3"/>
+      <c r="Z9" s="9"/>
+      <c r="AB9" s="5"/>
+      <c r="AC9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AD9" s="49">
+        <v>0.0015100000000000001</v>
+      </c>
+      <c r="AE9" s="32">
+        <v>0.00109</v>
+      </c>
+      <c r="AF9" s="23">
+        <v>0.00035599999999999998</v>
+      </c>
+      <c r="AG9" s="24">
+        <v>8.0499999999999992e-06</v>
+      </c>
+      <c r="AH9" s="45">
+        <v>7.5499999999999998e-11</v>
+      </c>
+      <c r="AI9" s="50" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="10" ht="14.25">
       <c r="B10" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C10" s="16">
         <v>5</v>
@@ -1547,9 +1814,9 @@
       <c r="G10" s="16">
         <v>5</v>
       </c>
-      <c r="J10" s="9"/>
+      <c r="J10" s="5"/>
       <c r="K10" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="L10" s="29">
         <v>0.022800000000000001</v>
@@ -1557,26 +1824,48 @@
       <c r="M10" s="29">
         <v>0.0137</v>
       </c>
-      <c r="N10" s="18">
+      <c r="N10" s="17">
         <v>0.0030000000000000001</v>
       </c>
-      <c r="O10" s="19">
+      <c r="O10" s="18">
         <v>3.4499999999999998e-05</v>
       </c>
-      <c r="P10" s="39">
+      <c r="P10" s="45">
         <v>9.4400000000000005e-11</v>
       </c>
-      <c r="Q10" s="41" t="s">
-        <v>28</v>
-      </c>
-      <c r="S10" s="4"/>
-      <c r="T10" s="31"/>
-      <c r="U10" s="4"/>
-      <c r="V10" s="4"/>
-      <c r="W10" s="4"/>
-      <c r="X10" s="4"/>
-      <c r="Y10" s="4"/>
-      <c r="Z10" s="10"/>
+      <c r="Q10" s="51" t="s">
+        <v>32</v>
+      </c>
+      <c r="S10" s="3"/>
+      <c r="T10" s="9"/>
+      <c r="U10" s="3"/>
+      <c r="V10" s="3"/>
+      <c r="W10" s="3"/>
+      <c r="X10" s="3"/>
+      <c r="Y10" s="3"/>
+      <c r="Z10" s="9"/>
+      <c r="AB10" s="5"/>
+      <c r="AC10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AD10" s="23">
+        <v>0.00086700000000000004</v>
+      </c>
+      <c r="AE10" s="23">
+        <v>0.00060599999999999998</v>
+      </c>
+      <c r="AF10" s="23">
+        <v>0.00018699999999999999</v>
+      </c>
+      <c r="AG10" s="24">
+        <v>4.0799999999999999e-06</v>
+      </c>
+      <c r="AH10" s="45">
+        <v>1.4700000000000002e-11</v>
+      </c>
+      <c r="AI10" s="52" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="11" ht="14.25">
       <c r="B11" s="1" t="s">
@@ -1597,7 +1886,7 @@
       <c r="G11" s="16">
         <v>5</v>
       </c>
-      <c r="J11" s="9"/>
+      <c r="J11" s="5"/>
       <c r="K11" s="1" t="s">
         <v>5</v>
       </c>
@@ -1616,80 +1905,111 @@
       <c r="P11" s="2">
         <v>0</v>
       </c>
-      <c r="Q11" s="42" t="s">
-        <v>29</v>
-      </c>
-      <c r="S11" s="4"/>
-      <c r="T11" s="31"/>
-      <c r="U11" s="4"/>
-      <c r="V11" s="4"/>
-      <c r="W11" s="4"/>
-      <c r="X11" s="4"/>
-      <c r="Y11" s="4"/>
-      <c r="Z11" s="10"/>
+      <c r="Q11" s="53" t="s">
+        <v>34</v>
+      </c>
+      <c r="S11" s="3"/>
+      <c r="T11" s="9"/>
+      <c r="U11" s="3"/>
+      <c r="V11" s="3"/>
+      <c r="W11" s="3"/>
+      <c r="X11" s="3"/>
+      <c r="Y11" s="3"/>
+      <c r="Z11" s="9"/>
+      <c r="AB11" s="5"/>
+      <c r="AC11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="AD11" s="23">
+        <v>0.00046900000000000002</v>
+      </c>
+      <c r="AE11" s="23">
+        <v>0.000321</v>
+      </c>
+      <c r="AF11" s="33">
+        <v>9.59e-05</v>
+      </c>
+      <c r="AG11" s="24">
+        <v>2.0499999999999999e-06</v>
+      </c>
+      <c r="AH11" s="45">
+        <v>6.0000000000000003e-12</v>
+      </c>
+      <c r="AI11" s="54" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="12" ht="14.25">
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="10"/>
-      <c r="L12" s="10"/>
-      <c r="M12" s="10"/>
-      <c r="N12" s="10"/>
-      <c r="O12" s="10"/>
-      <c r="P12" s="10"/>
-      <c r="S12" s="4"/>
-      <c r="T12" s="10"/>
-      <c r="U12" s="10"/>
-      <c r="V12" s="10"/>
-      <c r="W12" s="10"/>
-      <c r="X12" s="10"/>
-      <c r="Y12" s="10"/>
-      <c r="Z12" s="10"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="9"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="9"/>
+      <c r="O12" s="9"/>
+      <c r="P12" s="9"/>
+      <c r="S12" s="3"/>
+      <c r="T12" s="9"/>
+      <c r="U12" s="9"/>
+      <c r="V12" s="9"/>
+      <c r="W12" s="9"/>
+      <c r="X12" s="9"/>
+      <c r="Y12" s="9"/>
+      <c r="Z12" s="9"/>
     </row>
     <row r="13" ht="14.25">
-      <c r="A13" s="43"/>
-      <c r="B13" s="43"/>
-      <c r="C13" s="43"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="43"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="43"/>
-      <c r="H13" s="43"/>
-      <c r="I13" s="43"/>
-      <c r="J13" s="44"/>
-      <c r="K13" s="43"/>
-      <c r="L13" s="43"/>
-      <c r="M13" s="43"/>
-      <c r="N13" s="43"/>
-      <c r="O13" s="43"/>
-      <c r="P13" s="43"/>
-      <c r="Q13" s="43"/>
-      <c r="R13" s="43"/>
-      <c r="S13" s="43"/>
-      <c r="T13" s="43"/>
-      <c r="U13" s="43"/>
-      <c r="V13" s="43"/>
-      <c r="W13" s="43"/>
-      <c r="X13" s="43"/>
-      <c r="Y13" s="43"/>
-      <c r="Z13" s="43"/>
-      <c r="AA13" s="43"/>
+      <c r="A13" s="55"/>
+      <c r="B13" s="55"/>
+      <c r="C13" s="55"/>
+      <c r="D13" s="55"/>
+      <c r="E13" s="55"/>
+      <c r="F13" s="55"/>
+      <c r="G13" s="55"/>
+      <c r="H13" s="55"/>
+      <c r="I13" s="55"/>
+      <c r="J13" s="56"/>
+      <c r="K13" s="55"/>
+      <c r="L13" s="55"/>
+      <c r="M13" s="55"/>
+      <c r="N13" s="55"/>
+      <c r="O13" s="55"/>
+      <c r="P13" s="55"/>
+      <c r="Q13" s="55"/>
+      <c r="R13" s="55"/>
+      <c r="S13" s="55"/>
+      <c r="T13" s="55"/>
+      <c r="U13" s="55"/>
+      <c r="V13" s="55"/>
+      <c r="W13" s="55"/>
+      <c r="X13" s="55"/>
+      <c r="Y13" s="55"/>
+      <c r="Z13" s="55"/>
+      <c r="AA13" s="55"/>
+      <c r="AB13" s="55"/>
+      <c r="AC13" s="55"/>
+      <c r="AD13" s="55"/>
+      <c r="AE13" s="55"/>
+      <c r="AF13" s="55"/>
+      <c r="AG13" s="55"/>
+      <c r="AH13" s="55"/>
+      <c r="AI13" s="55"/>
+      <c r="AJ13" s="55"/>
     </row>
     <row r="14" ht="14.25">
-      <c r="B14" s="10"/>
-      <c r="Z14" s="10"/>
+      <c r="B14" s="9"/>
+      <c r="Z14" s="9"/>
     </row>
     <row r="15" ht="14.25">
-      <c r="A15" s="4"/>
+      <c r="A15" s="3"/>
       <c r="B15" t="s">
         <v>0</v>
       </c>
-      <c r="C15" s="9"/>
+      <c r="C15" s="5"/>
       <c r="D15" s="1" t="s">
         <v>1</v>
       </c>
@@ -1702,12 +2022,12 @@
       <c r="G15" s="2">
         <v>5</v>
       </c>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
       <c r="J15" t="s">
-        <v>3</v>
-      </c>
-      <c r="K15" s="9"/>
+        <v>36</v>
+      </c>
+      <c r="K15" s="5"/>
       <c r="L15" s="1" t="s">
         <v>4</v>
       </c>
@@ -1720,14 +2040,14 @@
       <c r="O15" s="2">
         <v>5</v>
       </c>
-      <c r="P15" s="4"/>
-      <c r="Q15" s="4"/>
-      <c r="R15" s="4"/>
-      <c r="S15" s="4"/>
-      <c r="T15" s="4" t="s">
+      <c r="P15" s="3"/>
+      <c r="Q15" s="3"/>
+      <c r="R15" s="3"/>
+      <c r="S15" s="3"/>
+      <c r="T15" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="U15" s="5"/>
+      <c r="U15" s="3"/>
       <c r="V15" s="1" t="s">
         <v>1</v>
       </c>
@@ -1740,72 +2060,111 @@
       <c r="Y15" s="2">
         <v>5</v>
       </c>
-      <c r="Z15" s="10"/>
+      <c r="Z15" s="9"/>
+      <c r="AB15" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="AC15" s="5"/>
+      <c r="AD15" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AE15" s="2">
+        <v>256</v>
+      </c>
+      <c r="AF15" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="AG15" s="2">
+        <v>5</v>
+      </c>
+      <c r="AH15" s="3"/>
+      <c r="AI15" s="3"/>
+      <c r="AJ15" s="3"/>
     </row>
     <row r="16" ht="14.25">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
-      <c r="M16" s="4"/>
-      <c r="N16" s="4"/>
-      <c r="O16" s="4"/>
-      <c r="P16" s="4"/>
-      <c r="Q16" s="4"/>
-      <c r="R16" s="4"/>
-      <c r="S16" s="4"/>
-      <c r="T16" s="4"/>
-      <c r="U16" s="4"/>
-      <c r="V16" s="4"/>
-      <c r="W16" s="4"/>
-      <c r="X16" s="4"/>
-      <c r="Y16" s="4"/>
-      <c r="Z16" s="10"/>
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
+      <c r="M16" s="3"/>
+      <c r="N16" s="3"/>
+      <c r="O16" s="3"/>
+      <c r="P16" s="3"/>
+      <c r="Q16" s="3"/>
+      <c r="R16" s="3"/>
+      <c r="S16" s="3"/>
+      <c r="T16" s="3"/>
+      <c r="U16" s="3"/>
+      <c r="V16" s="3"/>
+      <c r="W16" s="3"/>
+      <c r="X16" s="3"/>
+      <c r="Y16" s="3"/>
+      <c r="Z16" s="9"/>
+      <c r="AB16" s="3"/>
+      <c r="AC16" s="3"/>
+      <c r="AD16" s="3"/>
+      <c r="AE16" s="3"/>
+      <c r="AF16" s="3"/>
+      <c r="AG16" s="3"/>
+      <c r="AH16" s="3"/>
+      <c r="AI16" s="3"/>
+      <c r="AJ16" s="3"/>
     </row>
     <row r="17" ht="14.25">
-      <c r="A17" s="4"/>
+      <c r="A17" s="3"/>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
       <c r="D17" s="7" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
       <c r="G17" s="6"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
       <c r="K17" s="6"/>
       <c r="L17" s="6"/>
       <c r="M17" s="7" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N17" s="6"/>
       <c r="O17" s="6"/>
       <c r="P17" s="6"/>
-      <c r="Q17" s="4"/>
-      <c r="R17" s="4"/>
-      <c r="S17" s="4"/>
+      <c r="Q17" s="3"/>
+      <c r="R17" s="3"/>
+      <c r="S17" s="3"/>
       <c r="T17" s="6"/>
       <c r="U17" s="6"/>
       <c r="V17" s="7" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="W17" s="6"/>
       <c r="X17" s="6"/>
       <c r="Y17" s="6"/>
-      <c r="Z17" s="10"/>
+      <c r="Z17" s="9"/>
+      <c r="AB17" s="3"/>
+      <c r="AC17" s="6"/>
+      <c r="AD17" s="6"/>
+      <c r="AE17" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="AF17" s="6"/>
+      <c r="AG17" s="6"/>
+      <c r="AH17" s="6"/>
+      <c r="AI17" s="3"/>
+      <c r="AJ17" s="3"/>
     </row>
     <row r="18" ht="14.25">
-      <c r="A18" s="9"/>
+      <c r="A18" s="5"/>
       <c r="B18" s="1"/>
       <c r="C18" s="8">
         <v>1</v>
@@ -1822,60 +2181,79 @@
       <c r="G18" s="1">
         <v>16</v>
       </c>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="9"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="5"/>
       <c r="K18" s="1"/>
       <c r="L18" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="P18" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q18" s="4"/>
-      <c r="R18" s="4"/>
-      <c r="S18" s="9"/>
+        <v>14</v>
+      </c>
+      <c r="Q18" s="3"/>
+      <c r="R18" s="3"/>
+      <c r="S18" s="5"/>
       <c r="T18" s="1"/>
       <c r="U18" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="V18" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="W18" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="X18" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="Y18" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Z18" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="AB18" s="5"/>
+      <c r="AC18" s="1"/>
+      <c r="AD18" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="X18" s="1" t="s">
+      <c r="AE18" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="Y18" s="1" t="s">
+      <c r="AF18" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="Z18" s="17" t="s">
+      <c r="AG18" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="AH18" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="AI18" s="11"/>
+      <c r="AJ18" s="3"/>
     </row>
     <row r="19" ht="14.25">
-      <c r="A19" s="9"/>
+      <c r="A19" s="5"/>
       <c r="B19" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C19" s="45">
+        <v>16</v>
+      </c>
+      <c r="C19" s="57">
         <v>2.75</v>
       </c>
-      <c r="D19" s="46">
+      <c r="D19" s="58">
         <v>3</v>
       </c>
-      <c r="E19" s="45">
+      <c r="E19" s="57">
         <v>4.25</v>
       </c>
       <c r="F19" s="27">
@@ -1884,68 +2262,91 @@
       <c r="G19" s="16">
         <v>5</v>
       </c>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="9"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="5"/>
       <c r="K19" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="L19" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="M19" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="N19" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="O19" s="18">
+        <v>16</v>
+      </c>
+      <c r="L19" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M19" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N19" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="O19" s="17">
         <v>0.0030000000000000001</v>
       </c>
-      <c r="P19" s="19">
+      <c r="P19" s="18">
         <v>6.9999999999999994e-05</v>
       </c>
-      <c r="Q19" s="17" t="s">
+      <c r="Q19" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="R19" s="19"/>
+      <c r="S19" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="T19" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="U19" s="21">
+        <v>3.10546875</v>
+      </c>
+      <c r="V19" s="21">
+        <v>3.484375</v>
+      </c>
+      <c r="W19" s="21">
+        <v>4.0078125</v>
+      </c>
+      <c r="X19" s="21">
+        <v>4.83203125</v>
+      </c>
+      <c r="Y19" s="22">
+        <v>5</v>
+      </c>
+      <c r="Z19" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="AB19" s="5"/>
+      <c r="AC19" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R19" s="20"/>
-      <c r="S19" s="21" t="s">
-        <v>4</v>
-      </c>
-      <c r="T19" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="U19" s="22">
-        <v>3.10546875</v>
-      </c>
-      <c r="V19" s="22">
-        <v>3.484375</v>
-      </c>
-      <c r="W19" s="22">
-        <v>4.0078125</v>
-      </c>
-      <c r="X19" s="22">
-        <v>4.83203125</v>
-      </c>
-      <c r="Y19" s="23">
-        <v>5</v>
-      </c>
-      <c r="Z19" s="23" t="s">
-        <v>17</v>
-      </c>
+      <c r="AD19" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE19" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF19" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG19" s="23">
+        <v>0.00029100000000000003</v>
+      </c>
+      <c r="AH19" s="24">
+        <v>8.7299999999999994e-06</v>
+      </c>
+      <c r="AI19" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="AJ19" s="3"/>
     </row>
     <row r="20" ht="14.25">
-      <c r="A20" s="21"/>
+      <c r="A20" s="20"/>
       <c r="B20" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="C20" s="45">
+        <v>20</v>
+      </c>
+      <c r="C20" s="57">
         <v>2.375</v>
       </c>
-      <c r="D20" s="47">
+      <c r="D20" s="59">
         <v>3</v>
       </c>
-      <c r="E20" s="48">
+      <c r="E20" s="60">
         <v>5</v>
       </c>
       <c r="F20" s="16">
@@ -1954,49 +2355,71 @@
       <c r="G20" s="16">
         <v>5</v>
       </c>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="21"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="20"/>
       <c r="K20" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="L20" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="M20" s="17" t="s">
-        <v>15</v>
+        <v>20</v>
+      </c>
+      <c r="L20" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M20" s="10" t="s">
+        <v>17</v>
       </c>
       <c r="N20" s="29">
         <v>0.0112</v>
       </c>
-      <c r="O20" s="36">
+      <c r="O20" s="24">
         <v>0.00018200000000000001</v>
       </c>
-      <c r="P20" s="19">
+      <c r="P20" s="18">
         <v>3.6399999999999999e-06</v>
       </c>
       <c r="Q20" s="30" t="s">
-        <v>19</v>
-      </c>
-      <c r="R20" s="20"/>
-      <c r="S20"/>
-      <c r="T20" s="31"/>
-      <c r="U20" s="10"/>
-      <c r="V20" s="10"/>
-      <c r="W20" s="10"/>
-      <c r="X20" s="10"/>
-      <c r="Y20" s="10"/>
-      <c r="Z20" s="10"/>
+        <v>21</v>
+      </c>
+      <c r="R20" s="19"/>
+      <c r="T20" s="9"/>
+      <c r="U20" s="9"/>
+      <c r="V20" s="9"/>
+      <c r="W20" s="9"/>
+      <c r="X20" s="9"/>
+      <c r="Y20" s="9"/>
+      <c r="Z20" s="9"/>
+      <c r="AB20" s="20"/>
+      <c r="AC20" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="AD20" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE20" s="31" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF20" s="23">
+        <v>0.00043399999999999998</v>
+      </c>
+      <c r="AG20" s="33">
+        <v>1.49e-05</v>
+      </c>
+      <c r="AH20" s="18">
+        <v>3.72e-07</v>
+      </c>
+      <c r="AI20" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="AJ20" s="3"/>
     </row>
     <row r="21" ht="14.25">
-      <c r="A21" s="9"/>
+      <c r="A21" s="5"/>
       <c r="B21" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="C21" s="45">
+        <v>23</v>
+      </c>
+      <c r="C21" s="57">
         <v>2.75</v>
       </c>
-      <c r="D21" s="48">
+      <c r="D21" s="60">
         <v>5</v>
       </c>
       <c r="E21" s="16">
@@ -2008,50 +2431,72 @@
       <c r="G21" s="16">
         <v>5</v>
       </c>
-      <c r="H21" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="I21"/>
-      <c r="J21" s="5"/>
+      <c r="H21" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="J21" s="3"/>
       <c r="K21" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="L21" s="17" t="s">
-        <v>15</v>
+        <v>23</v>
+      </c>
+      <c r="L21" s="10" t="s">
+        <v>17</v>
       </c>
       <c r="M21" s="29">
         <v>0.065199999999999994</v>
       </c>
-      <c r="N21" s="18">
+      <c r="N21" s="17">
         <v>0.0020999999999999999</v>
       </c>
-      <c r="O21" s="19">
+      <c r="O21" s="18">
         <v>9.4599999999999992e-06</v>
       </c>
-      <c r="P21" s="19">
+      <c r="P21" s="18">
         <v>2.0100000000000001e-07</v>
       </c>
       <c r="Q21" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="R21" s="20"/>
-      <c r="S21" s="4"/>
-      <c r="T21" s="31"/>
-      <c r="U21" s="10"/>
-      <c r="V21" s="10"/>
-      <c r="W21" s="10"/>
-      <c r="X21" s="10"/>
-      <c r="Y21" s="10"/>
-      <c r="Z21" s="10"/>
+        <v>24</v>
+      </c>
+      <c r="R21" s="19"/>
+      <c r="S21" s="3"/>
+      <c r="T21" s="9"/>
+      <c r="U21" s="9"/>
+      <c r="V21" s="9"/>
+      <c r="W21" s="9"/>
+      <c r="X21" s="9"/>
+      <c r="Y21" s="9"/>
+      <c r="Z21" s="9"/>
+      <c r="AB21" s="5"/>
+      <c r="AC21" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="AD21" s="31" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE21" s="61">
+        <v>0.00083600000000000005</v>
+      </c>
+      <c r="AF21" s="62">
+        <v>5.6100000000000002e-05</v>
+      </c>
+      <c r="AG21" s="18">
+        <v>6.8500000000000001e-07</v>
+      </c>
+      <c r="AH21" s="18">
+        <v>1.7500000000000001e-08</v>
+      </c>
+      <c r="AI21" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="AJ21" s="3"/>
     </row>
     <row r="22" ht="14.25">
-      <c r="A22" s="21" t="s">
+      <c r="A22" s="20" t="s">
         <v>4</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C22" s="32">
+        <v>26</v>
+      </c>
+      <c r="C22" s="35">
         <v>5</v>
       </c>
       <c r="D22" s="16">
@@ -2066,15 +2511,15 @@
       <c r="G22" s="16">
         <v>5</v>
       </c>
-      <c r="H22" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="I22" s="4"/>
-      <c r="J22" s="31" t="s">
+      <c r="H22" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="I22" s="3"/>
+      <c r="J22" s="9" t="s">
         <v>4</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="L22" s="30">
         <v>0.10970000000000001</v>
@@ -2082,32 +2527,56 @@
       <c r="M22" s="29">
         <v>0.034799999999999998</v>
       </c>
-      <c r="N22" s="36">
+      <c r="N22" s="24">
         <v>0.00071299999999999998</v>
       </c>
-      <c r="O22" s="19">
+      <c r="O22" s="18">
         <v>5.1200000000000003e-07</v>
       </c>
-      <c r="P22" s="19">
+      <c r="P22" s="18">
         <v>1.1700000000000001e-08</v>
       </c>
-      <c r="Q22" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="R22" s="20"/>
-      <c r="S22"/>
-      <c r="T22" s="31"/>
-      <c r="U22" s="10"/>
-      <c r="V22" s="10"/>
-      <c r="W22" s="10"/>
-      <c r="X22" s="10"/>
-      <c r="Y22" s="10"/>
-      <c r="Z22" s="4"/>
+      <c r="Q22" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="R22" s="19"/>
+      <c r="T22" s="9"/>
+      <c r="U22" s="9"/>
+      <c r="V22" s="9"/>
+      <c r="W22" s="9"/>
+      <c r="X22" s="9"/>
+      <c r="Y22" s="9"/>
+      <c r="Z22" s="3"/>
+      <c r="AB22" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="AC22" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AD22" s="63">
+        <v>0.00096299999999999999</v>
+      </c>
+      <c r="AE22" s="64">
+        <v>0.000435</v>
+      </c>
+      <c r="AF22" s="33">
+        <v>1.8e-05</v>
+      </c>
+      <c r="AG22" s="18">
+        <v>3.4e-08</v>
+      </c>
+      <c r="AH22" s="45">
+        <v>9.0899999999999996e-10</v>
+      </c>
+      <c r="AI22" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="AJ22" s="3"/>
     </row>
     <row r="23" ht="14.25">
-      <c r="A23" s="9"/>
+      <c r="A23" s="5"/>
       <c r="B23" s="1" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C23" s="16">
         <v>5</v>
@@ -2124,11 +2593,11 @@
       <c r="G23" s="16">
         <v>5</v>
       </c>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="9"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="5"/>
       <c r="K23" s="1" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="L23" s="29">
         <v>0.061899999999999997</v>
@@ -2136,32 +2605,55 @@
       <c r="M23" s="29">
         <v>0.017100000000000001</v>
       </c>
-      <c r="N23" s="36">
+      <c r="N23" s="24">
         <v>0.00030800000000000001</v>
       </c>
-      <c r="O23" s="19">
+      <c r="O23" s="18">
         <v>2.9999999999999997e-08</v>
       </c>
-      <c r="P23" s="39">
+      <c r="P23" s="45">
         <v>7.0099999999999996e-10</v>
       </c>
-      <c r="Q23" s="40" t="s">
-        <v>26</v>
-      </c>
-      <c r="R23" s="20"/>
-      <c r="S23" s="4"/>
-      <c r="T23" s="31"/>
-      <c r="U23" s="4"/>
-      <c r="V23" s="4"/>
-      <c r="W23" s="4"/>
-      <c r="X23" s="4"/>
-      <c r="Y23" s="4"/>
-      <c r="Z23" s="10"/>
+      <c r="Q23" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="R23" s="19"/>
+      <c r="S23" s="3"/>
+      <c r="T23" s="9"/>
+      <c r="U23" s="3"/>
+      <c r="V23" s="3"/>
+      <c r="W23" s="3"/>
+      <c r="X23" s="3"/>
+      <c r="Y23" s="3"/>
+      <c r="Z23" s="9"/>
+      <c r="AB23" s="5"/>
+      <c r="AC23" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AD23" s="65">
+        <v>0.00063299999999999999</v>
+      </c>
+      <c r="AE23" s="23">
+        <v>0.00024800000000000001</v>
+      </c>
+      <c r="AF23" s="24">
+        <v>8.9700000000000005e-06</v>
+      </c>
+      <c r="AG23" s="18">
+        <v>1.8899999999999999e-09</v>
+      </c>
+      <c r="AH23" s="45">
+        <v>4.9499999999999997e-11</v>
+      </c>
+      <c r="AI23" s="48" t="s">
+        <v>30</v>
+      </c>
+      <c r="AJ23" s="3"/>
     </row>
     <row r="24" ht="14.25">
-      <c r="A24" s="9"/>
+      <c r="A24" s="5"/>
       <c r="B24" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C24" s="16">
         <v>5</v>
@@ -2178,11 +2670,11 @@
       <c r="G24" s="16">
         <v>5</v>
       </c>
-      <c r="H24" s="4"/>
-      <c r="I24" s="4"/>
-      <c r="J24" s="9"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="5"/>
       <c r="K24" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="L24" s="29">
         <v>0.025000000000000001</v>
@@ -2190,29 +2682,52 @@
       <c r="M24" s="29">
         <v>0.015699999999999999</v>
       </c>
-      <c r="N24" s="36">
+      <c r="N24" s="24">
         <v>0.000105</v>
       </c>
-      <c r="O24" s="19">
+      <c r="O24" s="18">
         <v>1.9599999999999998e-09</v>
       </c>
-      <c r="P24" s="39">
+      <c r="P24" s="45">
         <v>4.0399999999999997e-11</v>
       </c>
-      <c r="Q24" s="41" t="s">
-        <v>28</v>
-      </c>
-      <c r="S24" s="4"/>
-      <c r="T24" s="31"/>
-      <c r="U24" s="4"/>
-      <c r="V24" s="4"/>
-      <c r="W24" s="4"/>
-      <c r="X24" s="4"/>
-      <c r="Y24" s="4"/>
-      <c r="Z24" s="10"/>
+      <c r="Q24" s="51" t="s">
+        <v>32</v>
+      </c>
+      <c r="S24" s="3"/>
+      <c r="T24" s="9"/>
+      <c r="U24" s="3"/>
+      <c r="V24" s="3"/>
+      <c r="W24" s="3"/>
+      <c r="X24" s="3"/>
+      <c r="Y24" s="3"/>
+      <c r="Z24" s="9"/>
+      <c r="AB24" s="5"/>
+      <c r="AC24" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AD24" s="23">
+        <v>0.00038299999999999999</v>
+      </c>
+      <c r="AE24" s="23">
+        <v>0.000137</v>
+      </c>
+      <c r="AF24" s="24">
+        <v>4.5900000000000001e-06</v>
+      </c>
+      <c r="AG24" s="45">
+        <v>1.3799999999999999e-10</v>
+      </c>
+      <c r="AH24" s="45">
+        <v>2.89e-12</v>
+      </c>
+      <c r="AI24" s="51" t="s">
+        <v>33</v>
+      </c>
+      <c r="AJ24" s="3"/>
     </row>
     <row r="25" ht="14.25">
-      <c r="A25" s="9"/>
+      <c r="A25" s="5"/>
       <c r="B25" s="1" t="s">
         <v>5</v>
       </c>
@@ -2231,9 +2746,9 @@
       <c r="G25" s="16">
         <v>5</v>
       </c>
-      <c r="H25" s="4"/>
-      <c r="I25" s="4"/>
-      <c r="J25" s="9"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="5"/>
       <c r="K25" s="1" t="s">
         <v>5</v>
       </c>
@@ -2252,64 +2767,105 @@
       <c r="P25" s="2">
         <v>0</v>
       </c>
-      <c r="Q25" s="42" t="s">
-        <v>29</v>
-      </c>
-      <c r="R25" s="4"/>
-      <c r="S25" s="4"/>
-      <c r="T25" s="31"/>
-      <c r="U25" s="4"/>
-      <c r="V25" s="4"/>
-      <c r="W25" s="4"/>
-      <c r="X25" s="4"/>
-      <c r="Y25" s="4"/>
-      <c r="Z25" s="10"/>
+      <c r="Q25" s="53" t="s">
+        <v>34</v>
+      </c>
+      <c r="R25" s="3"/>
+      <c r="S25" s="3"/>
+      <c r="T25" s="9"/>
+      <c r="U25" s="3"/>
+      <c r="V25" s="3"/>
+      <c r="W25" s="3"/>
+      <c r="X25" s="3"/>
+      <c r="Y25" s="3"/>
+      <c r="Z25" s="9"/>
+      <c r="AB25" s="5"/>
+      <c r="AC25" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="AD25" s="23">
+        <v>0.000214</v>
+      </c>
+      <c r="AE25" s="33">
+        <v>7.2299999999999996e-05</v>
+      </c>
+      <c r="AF25" s="24">
+        <v>2.3300000000000001e-06</v>
+      </c>
+      <c r="AG25" s="45">
+        <v>2.37e-11</v>
+      </c>
+      <c r="AH25" s="45">
+        <v>2.9500000000000002e-12</v>
+      </c>
+      <c r="AI25" s="53" t="s">
+        <v>35</v>
+      </c>
+      <c r="AJ25" s="3"/>
     </row>
     <row r="26" ht="14.25">
-      <c r="S26" s="10"/>
-      <c r="T26" s="10"/>
-      <c r="U26" s="10"/>
-      <c r="V26" s="10"/>
-      <c r="W26" s="10"/>
-      <c r="X26" s="10"/>
-      <c r="Y26" s="10"/>
-      <c r="Z26" s="10"/>
+      <c r="S26" s="9"/>
+      <c r="T26" s="9"/>
+      <c r="U26" s="9"/>
+      <c r="V26" s="9"/>
+      <c r="W26" s="9"/>
+      <c r="X26" s="9"/>
+      <c r="Y26" s="9"/>
+      <c r="Z26" s="9"/>
+      <c r="AB26" s="3"/>
+      <c r="AC26" s="3"/>
+      <c r="AD26" s="3"/>
+      <c r="AE26" s="3"/>
+      <c r="AF26" s="3"/>
+      <c r="AG26" s="3"/>
+      <c r="AH26" s="3"/>
+      <c r="AI26" s="3"/>
+      <c r="AJ26" s="3"/>
     </row>
     <row r="27" ht="14.25">
-      <c r="A27" s="43"/>
-      <c r="B27" s="43"/>
-      <c r="C27" s="43"/>
-      <c r="D27" s="43"/>
-      <c r="E27" s="43"/>
-      <c r="F27" s="43"/>
-      <c r="G27" s="43"/>
-      <c r="H27" s="43"/>
-      <c r="I27" s="43"/>
-      <c r="J27" s="43"/>
-      <c r="K27" s="43"/>
-      <c r="L27" s="43"/>
-      <c r="M27" s="43"/>
-      <c r="N27" s="43"/>
-      <c r="O27" s="43"/>
-      <c r="P27" s="43"/>
-      <c r="Q27" s="43"/>
-      <c r="R27" s="43"/>
-      <c r="S27" s="43"/>
-      <c r="T27" s="43"/>
-      <c r="U27" s="43"/>
-      <c r="V27" s="43"/>
-      <c r="W27" s="43"/>
-      <c r="X27" s="43"/>
-      <c r="Y27" s="43"/>
-      <c r="Z27" s="43"/>
-      <c r="AA27" s="43"/>
+      <c r="A27" s="55"/>
+      <c r="B27" s="55"/>
+      <c r="C27" s="55"/>
+      <c r="D27" s="55"/>
+      <c r="E27" s="55"/>
+      <c r="F27" s="55"/>
+      <c r="G27" s="55"/>
+      <c r="H27" s="55"/>
+      <c r="I27" s="55"/>
+      <c r="J27" s="55"/>
+      <c r="K27" s="55"/>
+      <c r="L27" s="55"/>
+      <c r="M27" s="55"/>
+      <c r="N27" s="55"/>
+      <c r="O27" s="55"/>
+      <c r="P27" s="55"/>
+      <c r="Q27" s="55"/>
+      <c r="R27" s="55"/>
+      <c r="S27" s="55"/>
+      <c r="T27" s="55"/>
+      <c r="U27" s="55"/>
+      <c r="V27" s="55"/>
+      <c r="W27" s="55"/>
+      <c r="X27" s="55"/>
+      <c r="Y27" s="55"/>
+      <c r="Z27" s="55"/>
+      <c r="AA27" s="55"/>
+      <c r="AB27" s="55"/>
+      <c r="AC27" s="55"/>
+      <c r="AD27" s="55"/>
+      <c r="AE27" s="55"/>
+      <c r="AF27" s="55"/>
+      <c r="AG27" s="55"/>
+      <c r="AH27" s="55"/>
+      <c r="AI27" s="55"/>
+      <c r="AJ27" s="55"/>
     </row>
     <row r="29" ht="14.25">
-      <c r="A29" s="4"/>
-      <c r="B29" s="4" t="s">
+      <c r="A29" s="3"/>
+      <c r="B29" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C29" s="9"/>
+      <c r="C29" s="5"/>
       <c r="D29" s="1" t="s">
         <v>1</v>
       </c>
@@ -2322,12 +2878,12 @@
       <c r="G29" s="2">
         <v>5</v>
       </c>
-      <c r="H29" s="4"/>
-      <c r="I29" s="4"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
       <c r="J29" t="s">
-        <v>3</v>
-      </c>
-      <c r="K29" s="9"/>
+        <v>36</v>
+      </c>
+      <c r="K29" s="5"/>
       <c r="L29" s="1" t="s">
         <v>4</v>
       </c>
@@ -2340,12 +2896,12 @@
       <c r="O29" s="2">
         <v>5</v>
       </c>
-      <c r="P29" s="4"/>
-      <c r="S29" s="4"/>
-      <c r="T29" s="4" t="s">
+      <c r="P29" s="3"/>
+      <c r="S29" s="3"/>
+      <c r="T29" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="U29" s="5"/>
+      <c r="U29" s="3"/>
       <c r="V29" s="1" t="s">
         <v>1</v>
       </c>
@@ -2358,65 +2914,104 @@
       <c r="Y29" s="2">
         <v>5</v>
       </c>
+      <c r="AB29" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="AC29" s="5"/>
+      <c r="AD29" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AE29" s="2">
+        <v>512</v>
+      </c>
+      <c r="AF29" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="AG29" s="2">
+        <v>5</v>
+      </c>
+      <c r="AH29" s="3"/>
+      <c r="AI29" s="3"/>
+      <c r="AJ29" s="3"/>
     </row>
     <row r="30" ht="14.25">
-      <c r="A30" s="4"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
-      <c r="G30" s="4"/>
-      <c r="H30" s="4"/>
-      <c r="I30" s="4"/>
-      <c r="J30" s="4"/>
-      <c r="K30" s="4"/>
-      <c r="L30" s="4"/>
-      <c r="M30" s="4"/>
-      <c r="N30" s="4"/>
-      <c r="O30" s="4"/>
-      <c r="P30" s="4"/>
-      <c r="S30" s="4"/>
-      <c r="T30" s="4"/>
-      <c r="U30" s="4"/>
-      <c r="V30" s="4"/>
-      <c r="W30" s="4"/>
-      <c r="X30" s="4"/>
-      <c r="Y30" s="4"/>
+      <c r="A30" s="3"/>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+      <c r="K30" s="3"/>
+      <c r="L30" s="3"/>
+      <c r="M30" s="3"/>
+      <c r="N30" s="3"/>
+      <c r="O30" s="3"/>
+      <c r="P30" s="3"/>
+      <c r="S30" s="3"/>
+      <c r="T30" s="3"/>
+      <c r="U30" s="3"/>
+      <c r="V30" s="3"/>
+      <c r="W30" s="3"/>
+      <c r="X30" s="3"/>
+      <c r="Y30" s="3"/>
+      <c r="AB30" s="3"/>
+      <c r="AC30" s="3"/>
+      <c r="AD30" s="3"/>
+      <c r="AE30" s="3"/>
+      <c r="AF30" s="3"/>
+      <c r="AG30" s="3"/>
+      <c r="AH30" s="3"/>
+      <c r="AI30" s="3"/>
+      <c r="AJ30" s="3"/>
     </row>
     <row r="31" ht="14.25">
-      <c r="A31" s="4"/>
+      <c r="A31" s="3"/>
       <c r="B31" s="6"/>
       <c r="C31" s="6"/>
       <c r="D31" s="7" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E31" s="6"/>
       <c r="F31" s="6"/>
       <c r="G31" s="6"/>
-      <c r="H31" s="4"/>
-      <c r="I31" s="4"/>
-      <c r="J31" s="4"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3"/>
+      <c r="J31" s="3"/>
       <c r="K31" s="6"/>
       <c r="L31" s="6"/>
       <c r="M31" s="7" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N31" s="6"/>
       <c r="O31" s="6"/>
       <c r="P31" s="6"/>
-      <c r="S31" s="4"/>
+      <c r="S31" s="3"/>
       <c r="T31" s="6"/>
       <c r="U31" s="6"/>
       <c r="V31" s="7" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="W31" s="6"/>
       <c r="X31" s="6"/>
       <c r="Y31" s="6"/>
+      <c r="AB31" s="3"/>
+      <c r="AC31" s="6"/>
+      <c r="AD31" s="6"/>
+      <c r="AE31" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="AF31" s="6"/>
+      <c r="AG31" s="6"/>
+      <c r="AH31" s="6"/>
+      <c r="AI31" s="3"/>
+      <c r="AJ31" s="3"/>
     </row>
     <row r="32" ht="14.25">
-      <c r="A32" s="9"/>
+      <c r="A32" s="5"/>
       <c r="B32" s="1"/>
       <c r="C32" s="8">
         <v>1</v>
@@ -2433,58 +3028,77 @@
       <c r="G32" s="1">
         <v>16</v>
       </c>
-      <c r="H32" s="4"/>
-      <c r="I32" s="4"/>
-      <c r="J32" s="9"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3"/>
+      <c r="J32" s="5"/>
       <c r="K32" s="1"/>
       <c r="L32" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O32" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="P32" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="S32" s="9"/>
+        <v>14</v>
+      </c>
+      <c r="S32" s="5"/>
       <c r="T32" s="1"/>
       <c r="U32" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="V32" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="W32" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="X32" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="Y32" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Z32" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="AB32" s="5"/>
+      <c r="AC32" s="1"/>
+      <c r="AD32" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="X32" s="1" t="s">
+      <c r="AE32" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="Y32" s="1" t="s">
+      <c r="AF32" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="Z32" s="17" t="s">
+      <c r="AG32" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="AH32" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="AI32" s="11"/>
+      <c r="AJ32" s="3"/>
     </row>
     <row r="33" ht="14.25">
-      <c r="A33" s="9"/>
+      <c r="A33" s="5"/>
       <c r="B33" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C33" s="46">
+        <v>16</v>
+      </c>
+      <c r="C33" s="58">
         <v>2.75</v>
       </c>
-      <c r="D33" s="46">
+      <c r="D33" s="58">
         <v>3</v>
       </c>
-      <c r="E33" s="45">
+      <c r="E33" s="57">
         <v>4.25</v>
       </c>
       <c r="F33" s="27">
@@ -2493,229 +3107,305 @@
       <c r="G33" s="16">
         <v>5</v>
       </c>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="9"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="5"/>
       <c r="K33" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="L33" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="M33" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="N33" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="O33" s="18">
+        <v>16</v>
+      </c>
+      <c r="L33" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M33" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N33" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="O33" s="17">
         <v>0.0030000000000000001</v>
       </c>
-      <c r="P33" s="19">
+      <c r="P33" s="18">
         <v>6.9999999999999994e-05</v>
       </c>
-      <c r="Q33" s="17" t="s">
+      <c r="Q33" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="R33" s="19"/>
+      <c r="S33" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="T33" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="U33" s="21">
+        <v>3.7382811999999999</v>
+      </c>
+      <c r="V33" s="21">
+        <v>4.16015625</v>
+      </c>
+      <c r="W33" s="21">
+        <v>4.6796875</v>
+      </c>
+      <c r="X33" s="22">
+        <v>5</v>
+      </c>
+      <c r="Y33" s="22">
+        <v>5</v>
+      </c>
+      <c r="Z33" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="AB33" s="5"/>
+      <c r="AC33" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R33" s="20"/>
-      <c r="S33" s="21" t="s">
-        <v>4</v>
-      </c>
-      <c r="T33" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="U33" s="22">
-        <v>3.7382811999999999</v>
-      </c>
-      <c r="V33" s="22">
-        <v>4.16015625</v>
-      </c>
-      <c r="W33" s="22">
-        <v>4.6796875</v>
-      </c>
-      <c r="X33" s="23">
-        <v>5</v>
-      </c>
-      <c r="Y33" s="23">
-        <v>5</v>
-      </c>
-      <c r="Z33" s="23" t="s">
-        <v>17</v>
-      </c>
+      <c r="AD33" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE33" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF33" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG33" s="23">
+        <v>0.00029100000000000003</v>
+      </c>
+      <c r="AH33" s="24">
+        <v>8.7299999999999994e-06</v>
+      </c>
+      <c r="AI33" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="AJ33" s="3"/>
     </row>
     <row r="34" ht="14.25">
-      <c r="A34" s="21"/>
+      <c r="A34" s="20"/>
       <c r="B34" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C34" s="66">
+        <v>2.375</v>
+      </c>
+      <c r="D34" s="59">
+        <v>3</v>
+      </c>
+      <c r="E34" s="60">
+        <v>5</v>
+      </c>
+      <c r="F34" s="16">
+        <v>5</v>
+      </c>
+      <c r="G34" s="16">
+        <v>5</v>
+      </c>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="20"/>
+      <c r="K34" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L34" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M34" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N34" s="17">
+        <v>0.0089999999999999993</v>
+      </c>
+      <c r="O34" s="24">
+        <v>0.00018200000000000001</v>
+      </c>
+      <c r="P34" s="18">
+        <v>3.6399999999999999e-06</v>
+      </c>
+      <c r="Q34" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="R34" s="19"/>
+      <c r="T34" s="9"/>
+      <c r="AB34" s="20"/>
+      <c r="AC34" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="AD34" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE34" s="31" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF34" s="23">
+        <v>0.00038499999999999998</v>
+      </c>
+      <c r="AG34" s="67">
+        <v>1.49e-05</v>
+      </c>
+      <c r="AH34" s="18">
+        <v>3.72e-07</v>
+      </c>
+      <c r="AI34" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="AJ34" s="3"/>
+    </row>
+    <row r="35" ht="14.25">
+      <c r="A35" s="5"/>
+      <c r="B35" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C35" s="59">
+        <v>2.5625</v>
+      </c>
+      <c r="D35" s="60">
+        <v>5</v>
+      </c>
+      <c r="E35" s="16">
+        <v>5</v>
+      </c>
+      <c r="F35" s="16">
+        <v>5</v>
+      </c>
+      <c r="G35" s="16">
+        <v>5</v>
+      </c>
+      <c r="H35" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C34" s="49">
-        <v>2.375</v>
-      </c>
-      <c r="D34" s="47">
-        <v>3</v>
-      </c>
-      <c r="E34" s="48">
-        <v>5</v>
-      </c>
-      <c r="F34" s="16">
-        <v>5</v>
-      </c>
-      <c r="G34" s="16">
-        <v>5</v>
-      </c>
-      <c r="H34" s="4"/>
-      <c r="I34" s="4"/>
-      <c r="J34" s="21"/>
-      <c r="K34" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="L34" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="M34" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="N34" s="18">
-        <v>0.0089999999999999993</v>
-      </c>
-      <c r="O34" s="36">
-        <v>0.00018200000000000001</v>
-      </c>
-      <c r="P34" s="19">
-        <v>3.6399999999999999e-06</v>
-      </c>
-      <c r="Q34" s="30" t="s">
-        <v>19</v>
-      </c>
-      <c r="R34" s="20"/>
-      <c r="S34"/>
-      <c r="T34" s="31"/>
-      <c r="U34"/>
-      <c r="V34"/>
-      <c r="W34"/>
-      <c r="X34"/>
-      <c r="Y34"/>
-    </row>
-    <row r="35" ht="14.25">
-      <c r="A35" s="9"/>
-      <c r="B35" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="C35" s="47">
-        <v>2.5625</v>
-      </c>
-      <c r="D35" s="48">
-        <v>5</v>
-      </c>
-      <c r="E35" s="16">
-        <v>5</v>
-      </c>
-      <c r="F35" s="16">
-        <v>5</v>
-      </c>
-      <c r="G35" s="16">
-        <v>5</v>
-      </c>
-      <c r="H35" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="I35"/>
-      <c r="J35" s="5"/>
+      <c r="J35" s="3"/>
       <c r="K35" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="L35" s="17" t="s">
-        <v>15</v>
+        <v>23</v>
+      </c>
+      <c r="L35" s="10" t="s">
+        <v>17</v>
       </c>
       <c r="M35" s="29">
         <v>0.017399999999999999</v>
       </c>
-      <c r="N35" s="36">
+      <c r="N35" s="24">
         <v>0.00076099999999999996</v>
       </c>
-      <c r="O35" s="19">
+      <c r="O35" s="18">
         <v>9.4499999999999993e-06</v>
       </c>
-      <c r="P35" s="19">
+      <c r="P35" s="18">
         <v>2.0100000000000001e-07</v>
       </c>
       <c r="Q35" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="R35" s="20"/>
-      <c r="S35" s="4"/>
-      <c r="T35" s="31"/>
-      <c r="U35"/>
-      <c r="V35"/>
-      <c r="W35"/>
-      <c r="X35"/>
-      <c r="Y35"/>
+        <v>24</v>
+      </c>
+      <c r="R35" s="19"/>
+      <c r="S35" s="3"/>
+      <c r="T35" s="9"/>
+      <c r="AB35" s="5"/>
+      <c r="AC35" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="AD35" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE35" s="61">
+        <v>0.000272</v>
+      </c>
+      <c r="AF35" s="68">
+        <v>2.58e-05</v>
+      </c>
+      <c r="AG35" s="18">
+        <v>6.8500000000000001e-07</v>
+      </c>
+      <c r="AH35" s="18">
+        <v>1.7500000000000001e-08</v>
+      </c>
+      <c r="AI35" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="AJ35" s="3"/>
     </row>
     <row r="36" ht="14.25">
-      <c r="A36" s="21" t="s">
+      <c r="A36" s="20" t="s">
         <v>4</v>
       </c>
       <c r="B36" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C36" s="57">
+        <v>4.71875</v>
+      </c>
+      <c r="D36" s="27">
+        <v>5</v>
+      </c>
+      <c r="E36" s="16">
+        <v>5</v>
+      </c>
+      <c r="F36" s="16">
+        <v>5</v>
+      </c>
+      <c r="G36" s="16">
+        <v>5</v>
+      </c>
+      <c r="H36" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="I36" s="3"/>
+      <c r="J36" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="K36" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="L36" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M36" s="17">
+        <v>0.0035999999999999999</v>
+      </c>
+      <c r="N36" s="18">
+        <v>3.6300000000000001e-05</v>
+      </c>
+      <c r="O36" s="18">
+        <v>5.0999999999999999e-07</v>
+      </c>
+      <c r="P36" s="18">
+        <v>1.1700000000000001e-08</v>
+      </c>
+      <c r="Q36" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="C36" s="45">
-        <v>4.71875</v>
-      </c>
-      <c r="D36" s="27">
-        <v>5</v>
-      </c>
-      <c r="E36" s="16">
-        <v>5</v>
-      </c>
-      <c r="F36" s="16">
-        <v>5</v>
-      </c>
-      <c r="G36" s="16">
-        <v>5</v>
-      </c>
-      <c r="H36" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="I36" s="4"/>
-      <c r="J36" s="31" t="s">
+      <c r="R36" s="19"/>
+      <c r="T36" s="9"/>
+      <c r="AB36" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="K36" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="L36" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="M36" s="18">
-        <v>0.0035999999999999999</v>
-      </c>
-      <c r="N36" s="19">
-        <v>3.6300000000000001e-05</v>
-      </c>
-      <c r="O36" s="19">
-        <v>5.0999999999999999e-07</v>
-      </c>
-      <c r="P36" s="19">
-        <v>1.1700000000000001e-08</v>
-      </c>
-      <c r="Q36" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="R36" s="20"/>
-      <c r="S36"/>
-      <c r="T36" s="31"/>
-      <c r="U36"/>
-      <c r="V36"/>
-      <c r="W36"/>
-      <c r="X36"/>
-      <c r="Y36"/>
+      <c r="AC36" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AD36" s="31" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE36" s="69">
+        <v>2.8900000000000001e-05</v>
+      </c>
+      <c r="AF36" s="24">
+        <v>1.1200000000000001e-06</v>
+      </c>
+      <c r="AG36" s="18">
+        <v>3.3799999999999998e-08</v>
+      </c>
+      <c r="AH36" s="45">
+        <v>9.0899999999999996e-10</v>
+      </c>
+      <c r="AI36" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="AJ36" s="3"/>
     </row>
     <row r="37" ht="14.25">
-      <c r="A37" s="9"/>
+      <c r="A37" s="5"/>
       <c r="B37" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C37" s="32">
+        <v>29</v>
+      </c>
+      <c r="C37" s="35">
         <v>5</v>
       </c>
       <c r="D37" s="16">
@@ -2730,43 +3420,66 @@
       <c r="G37" s="16">
         <v>5</v>
       </c>
-      <c r="H37" s="4"/>
-      <c r="I37" s="4"/>
-      <c r="J37" s="9"/>
+      <c r="H37" s="3"/>
+      <c r="I37" s="3"/>
+      <c r="J37" s="5"/>
       <c r="K37" s="1" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="L37" s="29">
         <v>0.030599999999999999</v>
       </c>
-      <c r="M37" s="36">
+      <c r="M37" s="24">
         <v>0.000785</v>
       </c>
-      <c r="N37" s="19">
+      <c r="N37" s="18">
         <v>1.72e-06</v>
       </c>
-      <c r="O37" s="19">
+      <c r="O37" s="18">
         <v>2.9000000000000002e-08</v>
       </c>
-      <c r="P37" s="39">
+      <c r="P37" s="45">
         <v>7.0099999999999996e-10</v>
       </c>
-      <c r="Q37" s="40" t="s">
-        <v>26</v>
-      </c>
-      <c r="R37" s="20"/>
-      <c r="S37" s="4"/>
-      <c r="T37" s="31"/>
-      <c r="U37" s="4"/>
-      <c r="V37" s="4"/>
-      <c r="W37" s="4"/>
-      <c r="X37" s="4"/>
-      <c r="Y37" s="4"/>
+      <c r="Q37" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="R37" s="19"/>
+      <c r="S37" s="3"/>
+      <c r="T37" s="9"/>
+      <c r="U37" s="3"/>
+      <c r="V37" s="3"/>
+      <c r="W37" s="3"/>
+      <c r="X37" s="3"/>
+      <c r="Y37" s="3"/>
+      <c r="AB37" s="5"/>
+      <c r="AC37" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AD37" s="65">
+        <v>0.00015799999999999999</v>
+      </c>
+      <c r="AE37" s="24">
+        <v>8.1799999999999996e-06</v>
+      </c>
+      <c r="AF37" s="18">
+        <v>4.9999999999999998e-08</v>
+      </c>
+      <c r="AG37" s="18">
+        <v>1.8199999999999999e-09</v>
+      </c>
+      <c r="AH37" s="45">
+        <v>4.9499999999999997e-11</v>
+      </c>
+      <c r="AI37" s="48" t="s">
+        <v>30</v>
+      </c>
+      <c r="AJ37" s="3"/>
     </row>
     <row r="38" ht="14.25">
-      <c r="A38" s="9"/>
+      <c r="A38" s="5"/>
       <c r="B38" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C38" s="16">
         <v>5</v>
@@ -2783,41 +3496,64 @@
       <c r="G38" s="16">
         <v>5</v>
       </c>
-      <c r="H38" s="4"/>
-      <c r="I38" s="4"/>
-      <c r="J38" s="9"/>
+      <c r="H38" s="3"/>
+      <c r="I38" s="3"/>
+      <c r="J38" s="5"/>
       <c r="K38" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="L38" s="29">
         <v>0.0115</v>
       </c>
-      <c r="M38" s="36">
+      <c r="M38" s="24">
         <v>0.000242</v>
       </c>
-      <c r="N38" s="19">
+      <c r="N38" s="18">
         <v>8.42e-08</v>
       </c>
-      <c r="O38" s="19">
+      <c r="O38" s="18">
         <v>1.63e-09</v>
       </c>
-      <c r="P38" s="39">
+      <c r="P38" s="45">
         <v>4.0399999999999997e-11</v>
       </c>
-      <c r="Q38" s="41" t="s">
-        <v>28</v>
-      </c>
-      <c r="R38" s="10"/>
-      <c r="S38" s="4"/>
-      <c r="T38" s="31"/>
-      <c r="U38" s="4"/>
-      <c r="V38" s="4"/>
-      <c r="W38" s="4"/>
-      <c r="X38" s="4"/>
-      <c r="Y38" s="4"/>
+      <c r="Q38" s="51" t="s">
+        <v>32</v>
+      </c>
+      <c r="R38" s="9"/>
+      <c r="S38" s="3"/>
+      <c r="T38" s="9"/>
+      <c r="U38" s="3"/>
+      <c r="V38" s="3"/>
+      <c r="W38" s="3"/>
+      <c r="X38" s="3"/>
+      <c r="Y38" s="3"/>
+      <c r="AB38" s="5"/>
+      <c r="AC38" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AD38" s="67">
+        <v>9.0199999999999997e-05</v>
+      </c>
+      <c r="AE38" s="24">
+        <v>3.7400000000000002e-06</v>
+      </c>
+      <c r="AF38" s="18">
+        <v>2.4699999999999999e-09</v>
+      </c>
+      <c r="AG38" s="45">
+        <v>1.0300000000000001e-10</v>
+      </c>
+      <c r="AH38" s="45">
+        <v>3.4399999999999999e-12</v>
+      </c>
+      <c r="AI38" s="51" t="s">
+        <v>33</v>
+      </c>
+      <c r="AJ38" s="3"/>
     </row>
     <row r="39" ht="14.25">
-      <c r="A39" s="9"/>
+      <c r="A39" s="5"/>
       <c r="B39" s="1" t="s">
         <v>5</v>
       </c>
@@ -2836,9 +3572,9 @@
       <c r="G39" s="16">
         <v>5</v>
       </c>
-      <c r="H39" s="4"/>
-      <c r="I39" s="4"/>
-      <c r="J39" s="9"/>
+      <c r="H39" s="3"/>
+      <c r="I39" s="3"/>
+      <c r="J39" s="5"/>
       <c r="K39" s="1" t="s">
         <v>5</v>
       </c>
@@ -2857,72 +3593,115 @@
       <c r="P39" s="2">
         <v>0</v>
       </c>
-      <c r="Q39" s="42" t="s">
-        <v>29</v>
-      </c>
-      <c r="S39" s="4"/>
-      <c r="T39" s="31"/>
-      <c r="U39" s="4"/>
-      <c r="V39" s="4"/>
-      <c r="W39" s="4"/>
-      <c r="X39" s="4"/>
-      <c r="Y39" s="4"/>
+      <c r="Q39" s="53" t="s">
+        <v>34</v>
+      </c>
+      <c r="S39" s="3"/>
+      <c r="T39" s="9"/>
+      <c r="U39" s="3"/>
+      <c r="V39" s="3"/>
+      <c r="W39" s="3"/>
+      <c r="X39" s="3"/>
+      <c r="Y39" s="3"/>
+      <c r="AB39" s="5"/>
+      <c r="AC39" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="AD39" s="67">
+        <v>4.9799999999999998e-05</v>
+      </c>
+      <c r="AE39" s="24">
+        <v>1.9099999999999999e-06</v>
+      </c>
+      <c r="AF39" s="45">
+        <v>1.42e-10</v>
+      </c>
+      <c r="AG39" s="45">
+        <v>6.3100000000000004e-12</v>
+      </c>
+      <c r="AH39" s="45">
+        <v>2.69e-12</v>
+      </c>
+      <c r="AI39" s="53" t="s">
+        <v>35</v>
+      </c>
+      <c r="AJ39" s="3"/>
+    </row>
+    <row r="40" ht="14.25">
+      <c r="AB40" s="3"/>
+      <c r="AC40" s="3"/>
+      <c r="AD40" s="3"/>
+      <c r="AE40" s="3"/>
+      <c r="AF40" s="3"/>
+      <c r="AG40" s="3"/>
+      <c r="AH40" s="3"/>
+      <c r="AI40" s="3"/>
+      <c r="AJ40" s="3"/>
     </row>
     <row r="41" ht="14.25">
-      <c r="A41" s="43"/>
-      <c r="B41" s="43"/>
-      <c r="C41" s="43"/>
-      <c r="D41" s="43"/>
-      <c r="E41" s="43"/>
-      <c r="F41" s="43"/>
-      <c r="G41" s="43"/>
-      <c r="H41" s="43"/>
-      <c r="I41" s="43"/>
-      <c r="J41" s="43"/>
-      <c r="K41" s="43"/>
-      <c r="L41" s="43"/>
-      <c r="M41" s="43"/>
-      <c r="N41" s="43"/>
-      <c r="O41" s="43"/>
-      <c r="P41" s="43"/>
-      <c r="Q41" s="43"/>
-      <c r="R41" s="43"/>
-      <c r="S41" s="43"/>
-      <c r="T41" s="43"/>
-      <c r="U41" s="43"/>
-      <c r="V41" s="43"/>
-      <c r="W41" s="43"/>
-      <c r="X41" s="43"/>
-      <c r="Y41" s="43"/>
-      <c r="Z41" s="43"/>
-      <c r="AA41" s="43"/>
+      <c r="A41" s="55"/>
+      <c r="B41" s="55"/>
+      <c r="C41" s="55"/>
+      <c r="D41" s="55"/>
+      <c r="E41" s="55"/>
+      <c r="F41" s="55"/>
+      <c r="G41" s="55"/>
+      <c r="H41" s="55"/>
+      <c r="I41" s="55"/>
+      <c r="J41" s="55"/>
+      <c r="K41" s="55"/>
+      <c r="L41" s="55"/>
+      <c r="M41" s="55"/>
+      <c r="N41" s="55"/>
+      <c r="O41" s="55"/>
+      <c r="P41" s="55"/>
+      <c r="Q41" s="55"/>
+      <c r="R41" s="55"/>
+      <c r="S41" s="55"/>
+      <c r="T41" s="55"/>
+      <c r="U41" s="55"/>
+      <c r="V41" s="55"/>
+      <c r="W41" s="55"/>
+      <c r="X41" s="55"/>
+      <c r="Y41" s="55"/>
+      <c r="Z41" s="55"/>
+      <c r="AA41" s="55"/>
+      <c r="AB41" s="55"/>
+      <c r="AC41" s="55"/>
+      <c r="AD41" s="55"/>
+      <c r="AE41" s="55"/>
+      <c r="AF41" s="55"/>
+      <c r="AG41" s="55"/>
+      <c r="AH41" s="55"/>
+      <c r="AI41" s="55"/>
+      <c r="AJ41" s="55"/>
     </row>
     <row r="42" ht="14.25">
-      <c r="A42" s="4"/>
-      <c r="B42" s="4"/>
-      <c r="C42" s="4"/>
+      <c r="A42" s="3"/>
+      <c r="B42" s="3"/>
+      <c r="C42" s="3"/>
       <c r="D42" s="6"/>
       <c r="E42" s="6"/>
       <c r="F42" s="6"/>
       <c r="G42" s="6"/>
-      <c r="H42" s="4"/>
-      <c r="I42" s="4"/>
-      <c r="J42" s="4"/>
-      <c r="K42" s="4"/>
-      <c r="L42" s="4"/>
-      <c r="M42" s="4"/>
-      <c r="N42" s="4"/>
-      <c r="O42" s="4"/>
-      <c r="P42" s="4"/>
-      <c r="Q42" s="4"/>
-      <c r="R42" s="4"/>
+      <c r="H42" s="3"/>
+      <c r="I42" s="3"/>
+      <c r="J42" s="3"/>
+      <c r="K42" s="3"/>
+      <c r="L42" s="3"/>
+      <c r="M42" s="3"/>
+      <c r="N42" s="3"/>
+      <c r="O42" s="3"/>
+      <c r="P42" s="3"/>
+      <c r="Q42" s="3"/>
+      <c r="R42" s="3"/>
     </row>
     <row r="43" ht="14.25">
-      <c r="A43" s="4"/>
-      <c r="B43" s="4" t="s">
+      <c r="A43" s="3"/>
+      <c r="B43" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C43" s="9"/>
+      <c r="C43" s="5"/>
       <c r="D43" s="1" t="s">
         <v>1</v>
       </c>
@@ -2935,12 +3714,12 @@
       <c r="G43" s="2">
         <v>5</v>
       </c>
-      <c r="H43" s="4"/>
-      <c r="I43" s="4"/>
+      <c r="H43" s="3"/>
+      <c r="I43" s="3"/>
       <c r="J43" t="s">
-        <v>3</v>
-      </c>
-      <c r="K43" s="9"/>
+        <v>36</v>
+      </c>
+      <c r="K43" s="5"/>
       <c r="L43" s="1" t="s">
         <v>4</v>
       </c>
@@ -2953,14 +3732,14 @@
       <c r="O43" s="2">
         <v>5</v>
       </c>
-      <c r="P43" s="4"/>
-      <c r="Q43" s="4"/>
-      <c r="R43" s="4"/>
-      <c r="S43" s="4"/>
-      <c r="T43" s="4" t="s">
+      <c r="P43" s="3"/>
+      <c r="Q43" s="3"/>
+      <c r="R43" s="3"/>
+      <c r="S43" s="3"/>
+      <c r="T43" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="U43" s="5"/>
+      <c r="U43" s="3"/>
       <c r="V43" s="1" t="s">
         <v>1</v>
       </c>
@@ -2973,77 +3752,116 @@
       <c r="Y43" s="2">
         <v>5</v>
       </c>
+      <c r="AB43" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="AC43" s="5"/>
+      <c r="AD43" s="70" t="s">
+        <v>8</v>
+      </c>
+      <c r="AE43" s="2">
+        <v>1024</v>
+      </c>
+      <c r="AF43" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="AG43" s="2">
+        <v>5</v>
+      </c>
+      <c r="AH43" s="3"/>
+      <c r="AI43" s="3"/>
+      <c r="AJ43" s="3"/>
     </row>
     <row r="44" ht="14.25">
-      <c r="A44" s="4"/>
-      <c r="B44" s="4"/>
-      <c r="C44" s="4"/>
-      <c r="D44" s="4"/>
-      <c r="E44" s="4"/>
-      <c r="F44" s="4"/>
-      <c r="G44" s="4"/>
-      <c r="H44" s="4"/>
-      <c r="I44" s="4"/>
-      <c r="J44" s="4"/>
-      <c r="K44" s="4"/>
-      <c r="L44" s="4"/>
-      <c r="M44" s="4"/>
-      <c r="N44" s="4"/>
-      <c r="O44" s="4"/>
-      <c r="P44" s="4"/>
-      <c r="Q44" s="4"/>
-      <c r="R44" s="4"/>
-      <c r="S44" s="4"/>
-      <c r="T44" s="4"/>
-      <c r="U44" s="4"/>
-      <c r="V44" s="4"/>
-      <c r="W44" s="4"/>
-      <c r="X44" s="4"/>
-      <c r="Y44" s="4"/>
+      <c r="A44" s="3"/>
+      <c r="B44" s="3"/>
+      <c r="C44" s="3"/>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+      <c r="H44" s="3"/>
+      <c r="I44" s="3"/>
+      <c r="J44" s="3"/>
+      <c r="K44" s="3"/>
+      <c r="L44" s="3"/>
+      <c r="M44" s="3"/>
+      <c r="N44" s="3"/>
+      <c r="O44" s="3"/>
+      <c r="P44" s="3"/>
+      <c r="Q44" s="3"/>
+      <c r="R44" s="3"/>
+      <c r="S44" s="3"/>
+      <c r="T44" s="3"/>
+      <c r="U44" s="3"/>
+      <c r="V44" s="3"/>
+      <c r="W44" s="3"/>
+      <c r="X44" s="3"/>
+      <c r="Y44" s="3"/>
+      <c r="AB44" s="3"/>
+      <c r="AC44" s="3"/>
+      <c r="AD44" s="3"/>
+      <c r="AE44" s="3"/>
+      <c r="AF44" s="3"/>
+      <c r="AG44" s="3"/>
+      <c r="AH44" s="3"/>
+      <c r="AI44" s="3"/>
+      <c r="AJ44" s="3"/>
     </row>
     <row r="45" ht="14.25">
-      <c r="A45" s="4"/>
+      <c r="A45" s="3"/>
       <c r="B45" s="6"/>
       <c r="C45" s="6"/>
       <c r="D45" s="7" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E45" s="6"/>
       <c r="F45" s="6"/>
       <c r="G45" s="6"/>
-      <c r="H45" s="4"/>
-      <c r="I45" s="4"/>
-      <c r="J45" s="4"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="3"/>
+      <c r="J45" s="3"/>
       <c r="K45" s="6"/>
       <c r="L45" s="6"/>
       <c r="M45" s="7" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N45" s="6"/>
       <c r="O45" s="6"/>
       <c r="P45" s="6"/>
-      <c r="Q45" s="4"/>
-      <c r="R45" s="4"/>
-      <c r="S45" s="4"/>
+      <c r="Q45" s="3"/>
+      <c r="R45" s="3"/>
+      <c r="S45" s="3"/>
       <c r="T45" s="6"/>
       <c r="U45" s="6"/>
       <c r="V45" s="7" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="W45" s="6"/>
       <c r="X45" s="6"/>
       <c r="Y45" s="6"/>
+      <c r="AB45" s="3"/>
+      <c r="AC45" s="6"/>
+      <c r="AD45" s="6"/>
+      <c r="AE45" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="AF45" s="6"/>
+      <c r="AG45" s="6"/>
+      <c r="AH45" s="6"/>
+      <c r="AI45" s="3"/>
+      <c r="AJ45" s="3"/>
     </row>
     <row r="46" ht="14.25">
-      <c r="A46" s="9"/>
+      <c r="A46" s="5"/>
       <c r="B46" s="1"/>
-      <c r="C46" s="50">
+      <c r="C46" s="71">
         <v>1</v>
       </c>
       <c r="D46" s="8">
         <v>2</v>
       </c>
-      <c r="E46" s="50">
+      <c r="E46" s="71">
         <v>4</v>
       </c>
       <c r="F46" s="1">
@@ -3052,60 +3870,79 @@
       <c r="G46" s="1">
         <v>16</v>
       </c>
-      <c r="H46" s="4"/>
-      <c r="I46" s="4"/>
-      <c r="J46" s="9"/>
+      <c r="H46" s="3"/>
+      <c r="I46" s="3"/>
+      <c r="J46" s="5"/>
       <c r="K46" s="1"/>
       <c r="L46" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M46" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="N46" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O46" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="P46" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q46" s="51"/>
-      <c r="R46" s="4"/>
-      <c r="S46" s="9"/>
+        <v>14</v>
+      </c>
+      <c r="Q46" s="72"/>
+      <c r="R46" s="3"/>
+      <c r="S46" s="5"/>
       <c r="T46" s="1"/>
       <c r="U46" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="V46" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="W46" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="X46" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="Y46" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Z46" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="AB46" s="5"/>
+      <c r="AC46" s="1"/>
+      <c r="AD46" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="X46" s="1" t="s">
+      <c r="AE46" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="Y46" s="1" t="s">
+      <c r="AF46" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="Z46" s="17" t="s">
+      <c r="AG46" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="AH46" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="AI46" s="11"/>
+      <c r="AJ46" s="3"/>
     </row>
     <row r="47" ht="14.25">
-      <c r="A47" s="9"/>
-      <c r="B47" s="52" t="s">
-        <v>14</v>
-      </c>
-      <c r="C47" s="45">
+      <c r="A47" s="5"/>
+      <c r="B47" s="73" t="s">
+        <v>16</v>
+      </c>
+      <c r="C47" s="57">
         <v>2.75</v>
       </c>
-      <c r="D47" s="49">
+      <c r="D47" s="66">
         <v>3</v>
       </c>
-      <c r="E47" s="53">
+      <c r="E47" s="74">
         <v>4.5</v>
       </c>
       <c r="F47" s="16">
@@ -3114,251 +3951,368 @@
       <c r="G47" s="16">
         <v>5</v>
       </c>
-      <c r="H47" s="4"/>
-      <c r="I47" s="4"/>
-      <c r="J47" s="9"/>
+      <c r="H47" s="3"/>
+      <c r="I47" s="3"/>
+      <c r="J47" s="5"/>
       <c r="K47" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="L47" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="M47" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="N47" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="O47" s="18">
+        <v>16</v>
+      </c>
+      <c r="L47" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M47" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N47" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="O47" s="17">
         <v>0.0030000000000000001</v>
       </c>
-      <c r="P47" s="19">
+      <c r="P47" s="18">
         <v>6.9999999999999994e-05</v>
       </c>
-      <c r="Q47" s="17" t="s">
+      <c r="Q47" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="S47" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="T47" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="U47" s="21">
+        <v>4.296875</v>
+      </c>
+      <c r="V47" s="21">
+        <v>4.8515625</v>
+      </c>
+      <c r="W47" s="22">
+        <v>5</v>
+      </c>
+      <c r="X47" s="22">
+        <v>5</v>
+      </c>
+      <c r="Y47" s="22">
+        <v>5</v>
+      </c>
+      <c r="Z47" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="AB47" s="5"/>
+      <c r="AC47" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="S47" s="21" t="s">
+      <c r="AD47" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE47" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF47" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="AG47" s="23">
+        <v>0.00029100000000000003</v>
+      </c>
+      <c r="AH47" s="24">
+        <v>8.7299999999999994e-06</v>
+      </c>
+      <c r="AI47" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="AJ47" s="3"/>
+    </row>
+    <row r="48" ht="14.25">
+      <c r="A48" s="20"/>
+      <c r="B48" s="73" t="s">
+        <v>20</v>
+      </c>
+      <c r="C48" s="75">
+        <v>2.375</v>
+      </c>
+      <c r="D48" s="76">
+        <v>3</v>
+      </c>
+      <c r="E48" s="16">
+        <v>5</v>
+      </c>
+      <c r="F48" s="16">
+        <v>5</v>
+      </c>
+      <c r="G48" s="16">
+        <v>5</v>
+      </c>
+      <c r="H48" s="72"/>
+      <c r="I48" s="3"/>
+      <c r="J48" s="20"/>
+      <c r="K48" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L48" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M48" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N48" s="17">
+        <v>0.0089999999999999993</v>
+      </c>
+      <c r="O48" s="24">
+        <v>0.00018200000000000001</v>
+      </c>
+      <c r="P48" s="18">
+        <v>3.6399999999999999e-06</v>
+      </c>
+      <c r="Q48" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="S48" s="9"/>
+      <c r="AB48" s="20"/>
+      <c r="AC48" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="AD48" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE48" s="31" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF48" s="23">
+        <v>0.00038499999999999998</v>
+      </c>
+      <c r="AG48" s="67">
+        <v>1.49e-05</v>
+      </c>
+      <c r="AH48" s="18">
+        <v>3.72e-07</v>
+      </c>
+      <c r="AI48" s="30" t="s">
+        <v>22</v>
+      </c>
+      <c r="AJ48" s="3"/>
+    </row>
+    <row r="49" ht="14.25">
+      <c r="A49" s="5"/>
+      <c r="B49" s="73" t="s">
+        <v>23</v>
+      </c>
+      <c r="C49" s="76">
+        <v>2.5625</v>
+      </c>
+      <c r="D49" s="16">
+        <v>5</v>
+      </c>
+      <c r="E49" s="16">
+        <v>5</v>
+      </c>
+      <c r="F49" s="16">
+        <v>5</v>
+      </c>
+      <c r="G49" s="16">
+        <v>5</v>
+      </c>
+      <c r="H49" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="I49" s="19"/>
+      <c r="J49" s="3"/>
+      <c r="K49" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="L49" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M49" s="29">
+        <v>0.014999999999999999</v>
+      </c>
+      <c r="N49" s="24">
+        <v>0.00076099999999999996</v>
+      </c>
+      <c r="O49" s="18">
+        <v>9.4499999999999993e-06</v>
+      </c>
+      <c r="P49" s="18">
+        <v>2.0100000000000001e-07</v>
+      </c>
+      <c r="Q49" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="S49" s="3"/>
+      <c r="AB49" s="5"/>
+      <c r="AC49" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="AD49" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE49" s="61">
+        <v>0.00025300000000000002</v>
+      </c>
+      <c r="AF49" s="68">
+        <v>2.58e-05</v>
+      </c>
+      <c r="AG49" s="18">
+        <v>6.8500000000000001e-07</v>
+      </c>
+      <c r="AH49" s="18">
+        <v>1.7500000000000001e-08</v>
+      </c>
+      <c r="AI49" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="AJ49" s="3"/>
+    </row>
+    <row r="50" ht="14.25">
+      <c r="A50" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="T47" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="U47" s="22">
-        <v>4.296875</v>
-      </c>
-      <c r="V47" s="22">
-        <v>4.8515625</v>
-      </c>
-      <c r="W47" s="23">
-        <v>5</v>
-      </c>
-      <c r="X47" s="23">
-        <v>5</v>
-      </c>
-      <c r="Y47" s="23">
-        <v>5</v>
-      </c>
-      <c r="Z47" s="23" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="48" ht="14.25">
-      <c r="A48" s="21"/>
-      <c r="B48" s="52" t="s">
-        <v>18</v>
-      </c>
-      <c r="C48" s="54">
-        <v>2.375</v>
-      </c>
-      <c r="D48" s="55">
-        <v>3</v>
-      </c>
-      <c r="E48" s="16">
-        <v>5</v>
-      </c>
-      <c r="F48" s="16">
-        <v>5</v>
-      </c>
-      <c r="G48" s="16">
-        <v>5</v>
-      </c>
-      <c r="H48" s="51"/>
-      <c r="I48" s="4"/>
-      <c r="J48" s="21"/>
-      <c r="K48" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="L48" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="M48" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="N48" s="18">
-        <v>0.0089999999999999993</v>
-      </c>
-      <c r="O48" s="36">
-        <v>0.00018200000000000001</v>
-      </c>
-      <c r="P48" s="19">
-        <v>3.6399999999999999e-06</v>
-      </c>
-      <c r="Q48" s="30" t="s">
-        <v>19</v>
-      </c>
-      <c r="S48" s="31"/>
-    </row>
-    <row r="49" ht="14.25">
-      <c r="A49" s="9"/>
-      <c r="B49" s="52" t="s">
-        <v>20</v>
-      </c>
-      <c r="C49" s="55">
-        <v>2.5625</v>
-      </c>
-      <c r="D49" s="16">
-        <v>5</v>
-      </c>
-      <c r="E49" s="16">
-        <v>5</v>
-      </c>
-      <c r="F49" s="16">
-        <v>5</v>
-      </c>
-      <c r="G49" s="16">
-        <v>5</v>
-      </c>
-      <c r="H49" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="I49" s="20"/>
-      <c r="J49" s="5"/>
-      <c r="K49" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="L49" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="M49" s="56">
-        <v>0.014999999999999999</v>
-      </c>
-      <c r="N49" s="36">
-        <v>0.00076099999999999996</v>
-      </c>
-      <c r="O49" s="19">
-        <v>9.4499999999999993e-06</v>
-      </c>
-      <c r="P49" s="19">
-        <v>2.0100000000000001e-07</v>
-      </c>
-      <c r="Q49" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="S49" s="5"/>
-    </row>
-    <row r="50" ht="14.25">
-      <c r="A50" s="21" t="s">
+      <c r="B50" s="73" t="s">
+        <v>26</v>
+      </c>
+      <c r="C50" s="76">
+        <v>5</v>
+      </c>
+      <c r="D50" s="16">
+        <v>5</v>
+      </c>
+      <c r="E50" s="16">
+        <v>5</v>
+      </c>
+      <c r="F50" s="16">
+        <v>5</v>
+      </c>
+      <c r="G50" s="16">
+        <v>5</v>
+      </c>
+      <c r="H50" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="I50" s="77"/>
+      <c r="J50" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B50" s="52" t="s">
+      <c r="K50" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="L50" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M50" s="17">
+        <v>0.0022000000000000001</v>
+      </c>
+      <c r="N50" s="18">
+        <v>3.6399999999999997e-05</v>
+      </c>
+      <c r="O50" s="18">
+        <v>5.0999999999999999e-07</v>
+      </c>
+      <c r="P50" s="18">
+        <v>1.1700000000000001e-08</v>
+      </c>
+      <c r="Q50" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="C50" s="55">
-        <v>5</v>
-      </c>
-      <c r="D50" s="16">
-        <v>5</v>
-      </c>
-      <c r="E50" s="16">
-        <v>5</v>
-      </c>
-      <c r="F50" s="16">
-        <v>5</v>
-      </c>
-      <c r="G50" s="16">
-        <v>5</v>
-      </c>
-      <c r="H50" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="I50" s="57"/>
-      <c r="J50" s="31" t="s">
+      <c r="S50" s="9"/>
+      <c r="AB50" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="K50" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="L50" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="M50" s="18">
-        <v>0.0022000000000000001</v>
-      </c>
-      <c r="N50" s="19">
-        <v>3.6399999999999997e-05</v>
-      </c>
-      <c r="O50" s="19">
-        <v>5.0999999999999999e-07</v>
-      </c>
-      <c r="P50" s="19">
-        <v>1.1700000000000001e-08</v>
-      </c>
-      <c r="Q50" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="S50" s="31"/>
+      <c r="AC50" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AD50" s="31" t="s">
+        <v>17</v>
+      </c>
+      <c r="AE50" s="69">
+        <v>2.6699999999999998e-05</v>
+      </c>
+      <c r="AF50" s="24">
+        <v>1.1200000000000001e-06</v>
+      </c>
+      <c r="AG50" s="18">
+        <v>3.3799999999999998e-08</v>
+      </c>
+      <c r="AH50" s="45">
+        <v>9.0899999999999996e-10</v>
+      </c>
+      <c r="AI50" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="AJ50" s="3"/>
     </row>
     <row r="51" ht="14.25">
-      <c r="A51" s="9"/>
+      <c r="A51" s="5"/>
       <c r="B51" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C51" s="16">
+        <v>5</v>
+      </c>
+      <c r="D51" s="16">
+        <v>5</v>
+      </c>
+      <c r="E51" s="16">
+        <v>5</v>
+      </c>
+      <c r="F51" s="16">
+        <v>5</v>
+      </c>
+      <c r="G51" s="16">
+        <v>5</v>
+      </c>
+      <c r="H51" s="3"/>
+      <c r="I51" s="3"/>
+      <c r="J51" s="5"/>
+      <c r="K51" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L51" s="17">
+        <v>0.0038999999999999998</v>
+      </c>
+      <c r="M51" s="24">
+        <v>0.26444728792420652</v>
+      </c>
+      <c r="N51" s="18">
+        <v>1.7099999999999999e-06</v>
+      </c>
+      <c r="O51" s="18">
+        <v>2.9000000000000002e-08</v>
+      </c>
+      <c r="P51" s="45">
+        <v>7.0099999999999996e-10</v>
+      </c>
+      <c r="Q51" s="48" t="s">
         <v>25</v>
       </c>
-      <c r="C51" s="16">
-        <v>5</v>
-      </c>
-      <c r="D51" s="16">
-        <v>5</v>
-      </c>
-      <c r="E51" s="16">
-        <v>5</v>
-      </c>
-      <c r="F51" s="16">
-        <v>5</v>
-      </c>
-      <c r="G51" s="16">
-        <v>5</v>
-      </c>
-      <c r="H51" s="4"/>
-      <c r="I51" s="4"/>
-      <c r="J51" s="9"/>
-      <c r="K51" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="L51" s="18">
-        <v>0.0038999999999999998</v>
-      </c>
-      <c r="M51" s="36">
-        <v>0.26444728792420652</v>
-      </c>
-      <c r="N51" s="19">
-        <v>1.7099999999999999e-06</v>
-      </c>
-      <c r="O51" s="19">
-        <v>2.9000000000000002e-08</v>
-      </c>
-      <c r="P51" s="39">
-        <v>7.0099999999999996e-10</v>
-      </c>
-      <c r="Q51" s="40" t="s">
-        <v>26</v>
-      </c>
-      <c r="S51" s="5"/>
+      <c r="S51" s="3"/>
+      <c r="AB51" s="5"/>
+      <c r="AC51" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AD51" s="78">
+        <v>1.4600000000000001e-05</v>
+      </c>
+      <c r="AE51" s="24">
+        <v>1.26e-06</v>
+      </c>
+      <c r="AF51" s="18">
+        <v>4.9899999999999997e-08</v>
+      </c>
+      <c r="AG51" s="18">
+        <v>1.8199999999999999e-09</v>
+      </c>
+      <c r="AH51" s="45">
+        <v>4.9499999999999997e-11</v>
+      </c>
+      <c r="AI51" s="48" t="s">
+        <v>30</v>
+      </c>
+      <c r="AJ51" s="3"/>
     </row>
     <row r="52" ht="14.25">
-      <c r="A52" s="9"/>
+      <c r="A52" s="5"/>
       <c r="B52" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C52" s="16">
         <v>5</v>
@@ -3375,34 +4329,57 @@
       <c r="G52" s="16">
         <v>5</v>
       </c>
-      <c r="H52" s="4"/>
-      <c r="I52" s="4"/>
-      <c r="J52" s="9"/>
+      <c r="H52" s="3"/>
+      <c r="I52" s="3"/>
+      <c r="J52" s="5"/>
       <c r="K52" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="L52" s="36">
+        <v>31</v>
+      </c>
+      <c r="L52" s="24">
         <v>0.00051699999999999999</v>
       </c>
-      <c r="M52" s="19">
+      <c r="M52" s="18">
         <v>4.9171302741709417e-06</v>
       </c>
-      <c r="N52" s="19">
+      <c r="N52" s="18">
         <v>8.3599999999999994e-08</v>
       </c>
-      <c r="O52" s="19">
+      <c r="O52" s="18">
         <v>1.63e-09</v>
       </c>
-      <c r="P52" s="39">
+      <c r="P52" s="45">
         <v>4.0399999999999997e-11</v>
       </c>
-      <c r="Q52" s="41" t="s">
-        <v>28</v>
-      </c>
-      <c r="S52" s="5"/>
+      <c r="Q52" s="51" t="s">
+        <v>32</v>
+      </c>
+      <c r="S52" s="3"/>
+      <c r="AB52" s="5"/>
+      <c r="AC52" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AD52" s="24">
+        <v>2.5299999999999999e-06</v>
+      </c>
+      <c r="AE52" s="18">
+        <v>5.1200000000000002e-08</v>
+      </c>
+      <c r="AF52" s="18">
+        <v>2.45e-09</v>
+      </c>
+      <c r="AG52" s="45">
+        <v>1.0300000000000001e-10</v>
+      </c>
+      <c r="AH52" s="45">
+        <v>3.2500000000000001e-12</v>
+      </c>
+      <c r="AI52" s="51" t="s">
+        <v>33</v>
+      </c>
+      <c r="AJ52" s="3"/>
     </row>
     <row r="53" ht="14.25">
-      <c r="A53" s="9"/>
+      <c r="A53" s="5"/>
       <c r="B53" s="1" t="s">
         <v>5</v>
       </c>
@@ -3421,9 +4398,9 @@
       <c r="G53" s="16">
         <v>5</v>
       </c>
-      <c r="H53" s="4"/>
-      <c r="I53" s="4"/>
-      <c r="J53" s="9"/>
+      <c r="H53" s="3"/>
+      <c r="I53" s="3"/>
+      <c r="J53" s="5"/>
       <c r="K53" s="1" t="s">
         <v>5</v>
       </c>
@@ -3442,11 +4419,56 @@
       <c r="P53" s="2">
         <v>0</v>
       </c>
-      <c r="Q53" s="42" t="s">
-        <v>29</v>
-      </c>
-      <c r="R53" s="4"/>
-      <c r="S53" s="5"/>
+      <c r="Q53" s="53" t="s">
+        <v>34</v>
+      </c>
+      <c r="R53" s="3"/>
+      <c r="S53" s="3"/>
+      <c r="AB53" s="5"/>
+      <c r="AC53" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="AD53" s="24">
+        <v>1.06e-06</v>
+      </c>
+      <c r="AE53" s="18">
+        <v>2.3499999999999999e-09</v>
+      </c>
+      <c r="AF53" s="45">
+        <v>1.2999999999999999e-10</v>
+      </c>
+      <c r="AG53" s="45">
+        <v>6.3100000000000004e-12</v>
+      </c>
+      <c r="AH53" s="45">
+        <v>2.7799999999999999e-12</v>
+      </c>
+      <c r="AI53" s="53" t="s">
+        <v>35</v>
+      </c>
+      <c r="AJ53" s="3"/>
+    </row>
+    <row r="54" ht="14.25">
+      <c r="AB54" s="3"/>
+      <c r="AC54" s="3"/>
+      <c r="AD54" s="3"/>
+      <c r="AE54" s="3"/>
+      <c r="AF54" s="3"/>
+      <c r="AG54" s="3"/>
+      <c r="AH54" s="3"/>
+      <c r="AI54" s="3"/>
+      <c r="AJ54" s="3"/>
+    </row>
+    <row r="55" ht="14.25">
+      <c r="AB55"/>
+      <c r="AC55"/>
+      <c r="AD55"/>
+      <c r="AE55"/>
+      <c r="AF55"/>
+      <c r="AG55"/>
+      <c r="AH55"/>
+      <c r="AI55"/>
+      <c r="AJ55"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>